<commit_message>
updated after match 9
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D5A9EBFC-D456-4EE2-8D50-9C1FB57B558D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01F7BCD-A1FD-4C65-A0B1-A4259791D67E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="768" yWindow="768" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1152" yWindow="1152" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1096,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>59</v>
+        <v>219</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>1</v>
@@ -1117,16 +1117,16 @@
         <v>1</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>1</v>
@@ -1251,16 +1251,16 @@
         <v>1</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>62</v>
+        <v>32</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>35</v>
+        <v>22</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>28</v>
+        <v>148</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>1</v>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>9</v>
+        <v>55</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>1</v>
@@ -1385,16 +1385,16 @@
         <v>1</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>148</v>
+        <v>96</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>1</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>72</v>
+        <v>185</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>1</v>
@@ -1439,7 +1439,7 @@
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>80</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1677,7 +1677,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>44</v>
+        <v>177</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>1</v>
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>25</v>
+        <v>168</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>1</v>
@@ -1751,7 +1751,7 @@
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>98</v>
+        <v>122</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>1</v>
@@ -1811,7 +1811,7 @@
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>72</v>
+        <v>224</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>1</v>
@@ -1930,7 +1930,7 @@
         <v>0</v>
       </c>
       <c r="AC9" s="1">
-        <v>19</v>
+        <v>45</v>
       </c>
       <c r="AD9" s="1" t="s">
         <v>1</v>
@@ -2079,7 +2079,7 @@
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>114</v>
+        <v>155</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>1</v>
@@ -2109,7 +2109,7 @@
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>18</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2257,7 +2257,7 @@
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>118</v>
+        <v>189</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>1</v>
@@ -2287,7 +2287,7 @@
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>78</v>
+        <v>146</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>1</v>
@@ -2436,7 +2436,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>64</v>
+        <v>144</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>1</v>
@@ -2481,7 +2481,7 @@
         <v>0</v>
       </c>
       <c r="AH13" s="1">
-        <v>45</v>
+        <v>68</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>1</v>
@@ -2511,7 +2511,7 @@
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>134</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>475</v>
+        <v>546</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>1</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>584</v>
+        <v>773</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>1</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>531</v>
+        <v>623</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>1</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>454</v>
+        <v>694</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>1</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>810</v>
+        <v>890</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>1</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>910</v>
+        <v>1259</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>1</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>869</v>
+        <v>982</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>1</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>658</v>
+        <v>780</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 16
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0700913F-D003-4958-839D-60F94282E261}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A0C8F4-EDFC-415D-90A2-D508B0C71EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1051,7 +1051,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>278</v>
+        <v>454</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>123</v>
@@ -1096,7 +1096,7 @@
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>241</v>
+        <v>402</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>123</v>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>73</v>
+        <v>103</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
@@ -1260,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="S5" s="1">
-        <v>0</v>
+        <v>86</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>123</v>
@@ -1424,7 +1424,7 @@
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>193</v>
+        <v>312</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>123</v>
@@ -1617,7 +1617,7 @@
         <v>0</v>
       </c>
       <c r="N7" s="1">
-        <v>126</v>
+        <v>194</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>123</v>
@@ -1692,7 +1692,7 @@
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>358</v>
+        <v>387</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>207</v>
+        <v>291</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
@@ -1900,7 +1900,7 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>34</v>
+        <v>51</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
@@ -1945,7 +1945,7 @@
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>294</v>
+        <v>384</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -2109,7 +2109,7 @@
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>74</v>
+        <v>163</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2138,7 +2138,7 @@
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>176</v>
+        <v>211</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>123</v>
@@ -2168,7 +2168,7 @@
         <v>0</v>
       </c>
       <c r="S11" s="1">
-        <v>184</v>
+        <v>211</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>123</v>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>123</v>
@@ -2347,7 +2347,7 @@
         <v>0</v>
       </c>
       <c r="AH12" s="1">
-        <v>213</v>
+        <v>287</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>123</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>841</v>
+        <v>1017</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1225</v>
+        <v>1437</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>1258</v>
+        <v>1326</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>1131</v>
+        <v>1422</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>1004</v>
+        <v>1011</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>123</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>1576</v>
+        <v>1740</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>1906</v>
+        <v>2054</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>1648</v>
+        <v>1737</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 17
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35A0C8F4-EDFC-415D-90A2-D508B0C71EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{841ED367-2D6A-4685-9FE9-7A5E5551E061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1066,22 +1066,22 @@
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>111</v>
+        <v>16</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="M3" s="1">
         <v>0</v>
       </c>
       <c r="N3" s="1">
-        <v>269</v>
+        <v>145</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>123</v>
@@ -1102,31 +1102,31 @@
         <v>123</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>104</v>
+        <v>30</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>87</v>
+        <v>51</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>139</v>
+        <v>12</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>123</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>123</v>
@@ -1206,16 +1206,16 @@
         <v>123</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>48</v>
+        <v>111</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
       </c>
       <c r="N4" s="1">
-        <v>65</v>
+        <v>334</v>
       </c>
       <c r="O4" s="1" t="s">
         <v>123</v>
@@ -1236,31 +1236,31 @@
         <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
+        <v>184</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="1">
         <v>154</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="1">
-        <v>137</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
@@ -1281,31 +1281,31 @@
         <v>123</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>89</v>
+        <v>63</v>
       </c>
       <c r="AK4" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL4" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM4" s="1">
+        <v>163</v>
+      </c>
+      <c r="AN4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO4" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="AP4" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="AL4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AN4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO4" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="AP4" s="1" t="s">
-        <v>29</v>
-      </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>0</v>
+        <v>177</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1340,16 +1340,16 @@
         <v>123</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>76</v>
+        <v>48</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="M5" s="1">
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>0</v>
+        <v>69</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>123</v>
@@ -1370,31 +1370,31 @@
         <v>123</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>60</v>
+        <v>104</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>38</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>0</v>
+        <v>159</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>123</v>
@@ -1415,31 +1415,31 @@
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>107</v>
+        <v>89</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>312</v>
+        <v>0</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>73</v>
+        <v>90</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>23</v>
+        <v>29</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>122</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1474,10 +1474,10 @@
         <v>123</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
@@ -1498,37 +1498,37 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>108</v>
+        <v>154</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="AA6" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AB6" s="1">
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>56</v>
+        <v>137</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>123</v>
@@ -1549,22 +1549,22 @@
         <v>123</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>97</v>
+        <v>312</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="AP6" s="1" t="s">
         <v>23</v>
@@ -1573,7 +1573,7 @@
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>203</v>
+        <v>122</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1608,16 +1608,16 @@
         <v>123</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>38</v>
+        <v>84</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
       </c>
       <c r="N7" s="1">
-        <v>194</v>
+        <v>0</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>123</v>
@@ -1638,81 +1638,81 @@
         <v>123</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>108</v>
+        <v>38</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>105</v>
+        <v>20</v>
       </c>
       <c r="AA7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>142</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AF7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="AB7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE7" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF7" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>0</v>
+        <v>252</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>387</v>
+        <v>97</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AQ7" s="1">
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>125</v>
+        <v>203</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>83</v>
+        <v>100</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>24</v>
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>144</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
@@ -1736,22 +1736,22 @@
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>58</v>
+        <v>38</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="M8" s="1">
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>180</v>
+        <v>194</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>123</v>
@@ -1772,40 +1772,40 @@
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>86</v>
+        <v>50</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>168</v>
+        <v>235</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>31</v>
+        <v>105</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>88</v>
+        <v>52</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
@@ -1817,39 +1817,39 @@
         <v>123</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>81</v>
+        <v>33</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>104</v>
+        <v>387</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>45</v>
+        <v>108</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>173</v>
+        <v>289</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -1876,7 +1876,7 @@
         <v>123</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>102</v>
+        <v>58</v>
       </c>
       <c r="L9" s="1" t="s">
         <v>54</v>
@@ -1885,7 +1885,7 @@
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>132</v>
+        <v>180</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
@@ -1906,61 +1906,61 @@
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>19</v>
+        <v>113</v>
       </c>
       <c r="V9" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0</v>
+      </c>
+      <c r="X9" s="1">
+        <v>108</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AA9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>287</v>
+      </c>
+      <c r="AD9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE9" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF9" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="W9" s="1">
-        <v>0</v>
-      </c>
-      <c r="X9" s="1">
-        <v>111</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z9" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AB9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="1">
-        <v>74</v>
-      </c>
-      <c r="AD9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE9" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="AF9" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>384</v>
+        <v>0</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>116</v>
+        <v>81</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
       </c>
       <c r="AM9" s="1">
-        <v>282</v>
+        <v>104</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>123</v>
@@ -1980,10 +1980,10 @@
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
@@ -2010,16 +2010,16 @@
         <v>123</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>67</v>
+        <v>102</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>21</v>
+        <v>54</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>34</v>
+        <v>132</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>123</v>
@@ -2040,61 +2040,61 @@
         <v>123</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>212</v>
+        <v>168</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z10" s="1" t="s">
-        <v>70</v>
+        <v>79</v>
       </c>
       <c r="AA10" s="1" t="s">
-        <v>23</v>
+        <v>17</v>
       </c>
       <c r="AB10" s="1">
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>58</v>
+        <v>78</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>201</v>
+        <v>384</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="AK10" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="AL10" s="1">
         <v>0</v>
       </c>
       <c r="AM10" s="1">
-        <v>229</v>
+        <v>294</v>
       </c>
       <c r="AN10" s="1" t="s">
         <v>123</v>
@@ -2114,16 +2114,16 @@
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>119</v>
+        <v>109</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>239</v>
+        <v>0</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
@@ -2144,16 +2144,16 @@
         <v>123</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="M11" s="1">
         <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>48</v>
+        <v>142</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>123</v>
@@ -2174,61 +2174,61 @@
         <v>123</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>74</v>
+        <v>111</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>96</v>
+        <v>70</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>150</v>
+        <v>58</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AF11" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AG11" s="1">
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>248</v>
+        <v>201</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>72</v>
+        <v>122</v>
       </c>
       <c r="AK11" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="AL11" s="1">
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>306</v>
+        <v>229</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>123</v>
@@ -2243,21 +2243,21 @@
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>166</v>
+        <v>282</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>100</v>
+        <v>119</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>140</v>
+        <v>296</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>123</v>
@@ -2308,16 +2308,16 @@
         <v>123</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>78</v>
+        <v>95</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>176</v>
+        <v>212</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
@@ -2332,7 +2332,7 @@
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
@@ -2353,16 +2353,16 @@
         <v>123</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>42</v>
+        <v>306</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
@@ -2377,7 +2377,7 @@
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>197</v>
+        <v>201</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2436,7 +2436,7 @@
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>43</v>
+        <v>67</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>123</v>
@@ -2466,7 +2466,7 @@
         <v>0</v>
       </c>
       <c r="AC13" s="1">
-        <v>142</v>
+        <v>218</v>
       </c>
       <c r="AD13" s="1" t="s">
         <v>123</v>
@@ -2481,22 +2481,22 @@
         <v>0</v>
       </c>
       <c r="AH13" s="1">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ13" s="1" t="s">
-        <v>63</v>
+        <v>53</v>
       </c>
       <c r="AK13" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="AL13" s="1">
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>159</v>
+        <v>42</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>123</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>1017</v>
+        <v>1078</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2540,7 +2540,7 @@
         <v>0</v>
       </c>
       <c r="I14" s="1">
-        <v>1437</v>
+        <v>1447</v>
       </c>
       <c r="J14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>1326</v>
+        <v>1600</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>1422</v>
+        <v>1450</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1355</v>
+        <v>1511</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>1011</v>
+        <v>1356</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>123</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>1740</v>
+        <v>1753</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>2054</v>
+        <v>2078</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>1737</v>
+        <v>2025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 18
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{841ED367-2D6A-4685-9FE9-7A5E5551E061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9425C5E-1E47-4BCA-8DE7-4B8C6573A380}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1081,7 +1081,7 @@
         <v>0</v>
       </c>
       <c r="N3" s="1">
-        <v>145</v>
+        <v>275</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>123</v>
@@ -1117,16 +1117,16 @@
         <v>123</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>51</v>
+        <v>96</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>12</v>
+        <v>261</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>123</v>
@@ -1156,7 +1156,7 @@
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>144</v>
+        <v>181</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>123</v>
@@ -1236,31 +1236,31 @@
         <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>78</v>
+        <v>104</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>184</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>96</v>
+        <v>87</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
@@ -1290,36 +1290,36 @@
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>177</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>123</v>
@@ -1349,7 +1349,7 @@
         <v>0</v>
       </c>
       <c r="N5" s="1">
-        <v>69</v>
+        <v>111</v>
       </c>
       <c r="O5" s="1" t="s">
         <v>123</v>
@@ -1370,31 +1370,31 @@
         <v>123</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>0</v>
+        <v>181</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>159</v>
+        <v>217</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>123</v>
@@ -1430,24 +1430,24 @@
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>0</v>
+        <v>219</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -1498,7 +1498,7 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>4</v>
+        <v>32</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
@@ -1564,30 +1564,30 @@
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>122</v>
+        <v>239</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
       </c>
       <c r="D7" s="1">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>123</v>
@@ -1668,16 +1668,16 @@
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>115</v>
+        <v>52</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>252</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
@@ -1698,7 +1698,7 @@
         <v>123</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="AP7" s="1" t="s">
         <v>23</v>
@@ -1707,21 +1707,21 @@
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>203</v>
+        <v>122</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
         <v>24</v>
-      </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>144</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
@@ -1802,10 +1802,10 @@
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>52</v>
+        <v>88</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
@@ -1832,16 +1832,16 @@
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>289</v>
+        <v>203</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1936,16 +1936,16 @@
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>88</v>
+        <v>115</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>0</v>
+        <v>265</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -1966,16 +1966,16 @@
         <v>123</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>64</v>
+        <v>108</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="AQ9" s="1">
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>147</v>
+        <v>289</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2064,7 +2064,7 @@
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>78</v>
+        <v>108</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
@@ -2100,16 +2100,16 @@
         <v>123</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>117</v>
+        <v>64</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>40</v>
+        <v>54</v>
       </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>163</v>
+        <v>147</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
@@ -2189,16 +2189,16 @@
         <v>123</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>58</v>
+        <v>20</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
@@ -2234,16 +2234,16 @@
         <v>123</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>35</v>
+        <v>117</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="AQ11" s="1">
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>282</v>
+        <v>163</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2323,16 +2323,16 @@
         <v>123</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AB12" s="1">
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>111</v>
+        <v>58</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
@@ -2368,16 +2368,16 @@
         <v>123</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>120</v>
+        <v>35</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="AQ12" s="1">
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>201</v>
+        <v>282</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="D14" s="1">
-        <v>1078</v>
+        <v>1150</v>
       </c>
       <c r="E14" s="1" t="s">
         <v>123</v>
@@ -2555,7 +2555,7 @@
         <v>0</v>
       </c>
       <c r="N14" s="1">
-        <v>1600</v>
+        <v>1772</v>
       </c>
       <c r="O14" s="1" t="s">
         <v>123</v>
@@ -2570,7 +2570,7 @@
         <v>0</v>
       </c>
       <c r="S14" s="1">
-        <v>1450</v>
+        <v>1478</v>
       </c>
       <c r="T14" s="1" t="s">
         <v>123</v>
@@ -2585,7 +2585,7 @@
         <v>0</v>
       </c>
       <c r="X14" s="1">
-        <v>1511</v>
+        <v>1508</v>
       </c>
       <c r="Y14" s="1" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
         <v>0</v>
       </c>
       <c r="AC14" s="1">
-        <v>1356</v>
+        <v>1607</v>
       </c>
       <c r="AD14" s="1" t="s">
         <v>123</v>
@@ -2615,7 +2615,7 @@
         <v>0</v>
       </c>
       <c r="AH14" s="1">
-        <v>1753</v>
+        <v>1766</v>
       </c>
       <c r="AI14" s="1" t="s">
         <v>123</v>
@@ -2630,7 +2630,7 @@
         <v>0</v>
       </c>
       <c r="AM14" s="1">
-        <v>2078</v>
+        <v>2117</v>
       </c>
       <c r="AN14" s="1" t="s">
         <v>123</v>
@@ -2645,7 +2645,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>2025</v>
+        <v>2105</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 20
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30FF90BC-9D18-417A-B42B-D40EEE3EB64C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0EEC387-F32A-4301-9CBB-795D9BF9831C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3000" yWindow="3000" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1151,7 +1151,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>242</v>
+        <v>281</v>
       </c>
       <c r="AI3" t="s">
         <v>123</v>
@@ -1240,7 +1240,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>79</v>
+        <v>97</v>
       </c>
       <c r="T4" t="s">
         <v>123</v>
@@ -1285,7 +1285,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>112</v>
+        <v>125</v>
       </c>
       <c r="AI4" t="s">
         <v>123</v>
@@ -1419,7 +1419,7 @@
         <v>0</v>
       </c>
       <c r="AH5">
-        <v>137</v>
+        <v>208</v>
       </c>
       <c r="AI5" t="s">
         <v>123</v>
@@ -1568,7 +1568,7 @@
         <v>0</v>
       </c>
       <c r="AM6">
-        <v>312</v>
+        <v>439</v>
       </c>
       <c r="AN6" t="s">
         <v>123</v>
@@ -1642,7 +1642,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>86</v>
+        <v>235</v>
       </c>
       <c r="T7" t="s">
         <v>123</v>
@@ -1880,7 +1880,7 @@
         <v>0</v>
       </c>
       <c r="I9">
-        <v>291</v>
+        <v>381</v>
       </c>
       <c r="J9" t="s">
         <v>123</v>
@@ -1910,7 +1910,7 @@
         <v>0</v>
       </c>
       <c r="S9">
-        <v>51</v>
+        <v>69</v>
       </c>
       <c r="T9" t="s">
         <v>123</v>
@@ -2014,7 +2014,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>23</v>
+        <v>69</v>
       </c>
       <c r="J10" t="s">
         <v>123</v>
@@ -2148,7 +2148,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>211</v>
+        <v>235</v>
       </c>
       <c r="J11" t="s">
         <v>123</v>
@@ -2178,7 +2178,7 @@
         <v>0</v>
       </c>
       <c r="S11">
-        <v>211</v>
+        <v>287</v>
       </c>
       <c r="T11" t="s">
         <v>123</v>
@@ -2193,7 +2193,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>111</v>
+        <v>247</v>
       </c>
       <c r="Y11" t="s">
         <v>123</v>
@@ -2253,7 +2253,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>163</v>
+        <v>215</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2282,7 +2282,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>140</v>
+        <v>294</v>
       </c>
       <c r="J12" t="s">
         <v>123</v>
@@ -2327,7 +2327,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>212</v>
+        <v>291</v>
       </c>
       <c r="Y12" t="s">
         <v>123</v>
@@ -2552,7 +2552,7 @@
       </c>
       <c r="I14">
         <f>SUM(I3:I13)</f>
-        <v>1478</v>
+        <v>1792</v>
       </c>
       <c r="J14" t="s">
         <v>123</v>
@@ -2584,7 +2584,7 @@
       </c>
       <c r="S14">
         <f>SUM(S3:S13)</f>
-        <v>1504</v>
+        <v>1765</v>
       </c>
       <c r="T14" t="s">
         <v>123</v>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="X14">
         <f>SUM(X3:X13)</f>
-        <v>1594</v>
+        <v>1809</v>
       </c>
       <c r="Y14" t="s">
         <v>123</v>
@@ -2632,7 +2632,7 @@
       </c>
       <c r="AH14">
         <f>SUM(AH3:AH13)</f>
-        <v>1828</v>
+        <v>1951</v>
       </c>
       <c r="AI14" t="s">
         <v>123</v>
@@ -2648,7 +2648,7 @@
       </c>
       <c r="AM14">
         <f>SUM(AM3:AM13)</f>
-        <v>2314</v>
+        <v>2441</v>
       </c>
       <c r="AN14" t="s">
         <v>123</v>
@@ -2664,7 +2664,7 @@
       </c>
       <c r="AR14">
         <f>SUM(AR3:AR13)</f>
-        <v>2460</v>
+        <v>2512</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 24
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{50892927-91B2-432B-845E-0DE70E476D25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE742CC-8446-46AF-88CC-051601248765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3348" yWindow="3348" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2592" yWindow="2028" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="400" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="125">
   <si>
     <t>Aizen</t>
   </si>
@@ -403,6 +403,9 @@
   </si>
   <si>
     <t/>
+  </si>
+  <si>
+    <t>Navdeep Saini</t>
   </si>
 </sst>
 </file>
@@ -780,7 +783,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AR14"/>
+  <dimension ref="A1:AR15"/>
   <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:44" x14ac:dyDescent="0.3">
@@ -1113,31 +1116,31 @@
         <v>123</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>300</v>
+        <v>268</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>87</v>
+        <v>42</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>159</v>
+        <v>217</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>123</v>
@@ -1173,21 +1176,21 @@
         <v>123</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>55</v>
+        <v>124</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>238</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>29</v>
@@ -1196,22 +1199,22 @@
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>146</v>
+        <v>40</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>121</v>
+        <v>37</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>470</v>
+        <v>160</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
@@ -1262,16 +1265,16 @@
         <v>123</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>217</v>
+        <v>189</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
@@ -1292,60 +1295,60 @@
         <v>123</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>107</v>
+        <v>63</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="AL4" s="1">
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>512</v>
+        <v>165</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>64</v>
+        <v>90</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>260</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
+        <v>171</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>103</v>
+        <v>470</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>123</v>
@@ -1366,16 +1369,16 @@
         <v>123</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>18</v>
+        <v>68</v>
       </c>
       <c r="Q5" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="R5" s="1">
         <v>0</v>
       </c>
       <c r="S5" s="1">
-        <v>95</v>
+        <v>0</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>123</v>
@@ -1396,90 +1399,90 @@
         <v>123</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>189</v>
+        <v>170</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>43</v>
+        <v>97</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AG5" s="1">
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>125</v>
+        <v>243</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>63</v>
+        <v>89</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>165</v>
+        <v>0</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>0</v>
+        <v>256</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>100</v>
+        <v>25</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
       </c>
       <c r="D6" s="1">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="E6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>26</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>241</v>
+        <v>103</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>123</v>
@@ -1500,37 +1503,37 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>77</v>
+        <v>112</v>
       </c>
       <c r="Q6" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="R6" s="1">
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>235</v>
+        <v>132</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>78</v>
+        <v>69</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>181</v>
+        <v>300</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>79</v>
+        <v>96</v>
       </c>
       <c r="AA6" s="1" t="s">
         <v>17</v>
@@ -1539,60 +1542,60 @@
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>170</v>
+        <v>351</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>97</v>
+        <v>88</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="AG6" s="1">
         <v>0</v>
       </c>
       <c r="AH6" s="1">
-        <v>243</v>
+        <v>220</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>89</v>
+        <v>107</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>0</v>
+        <v>512</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>256</v>
+        <v>238</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>25</v>
+        <v>36</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1">
         <v>0</v>
@@ -1604,16 +1607,16 @@
         <v>123</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>66</v>
+        <v>26</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>61</v>
+        <v>241</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>123</v>
@@ -1634,52 +1637,52 @@
         <v>123</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>68</v>
+        <v>39</v>
       </c>
       <c r="Q7" s="1" t="s">
-        <v>29</v>
+        <v>40</v>
       </c>
       <c r="R7" s="1">
         <v>0</v>
       </c>
       <c r="S7" s="1">
-        <v>0</v>
+        <v>160</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>41</v>
+        <v>78</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>270</v>
+        <v>181</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="AA7" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB7" s="1">
         <v>0</v>
       </c>
       <c r="AC7" s="1">
-        <v>142</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="AF7" s="1" t="s">
         <v>15</v>
@@ -1688,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>208</v>
+        <v>145</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
@@ -1723,31 +1726,31 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>36</v>
+        <v>65</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>146</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>75</v>
+        <v>66</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>24</v>
+        <v>40</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>0</v>
+        <v>61</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
@@ -1768,61 +1771,61 @@
         <v>123</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>112</v>
+        <v>28</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>132</v>
+        <v>187</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>60</v>
+        <v>41</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>38</v>
+        <v>270</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>96</v>
+        <v>51</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>351</v>
+        <v>20</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>52</v>
+        <v>32</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>40</v>
+        <v>15</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>0</v>
+        <v>210</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
@@ -1843,16 +1846,16 @@
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>73</v>
+        <v>64</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>186</v>
+        <v>260</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
@@ -1872,16 +1875,16 @@
         <v>123</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>75</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
@@ -1902,55 +1905,55 @@
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>39</v>
+        <v>77</v>
       </c>
       <c r="Q9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R9" s="1">
+        <v>0</v>
+      </c>
+      <c r="S9" s="1">
+        <v>240</v>
+      </c>
+      <c r="T9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="V9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="W9" s="1">
+        <v>0</v>
+      </c>
+      <c r="X9" s="1">
+        <v>38</v>
+      </c>
+      <c r="Y9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z9" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>84</v>
+      </c>
+      <c r="AD9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE9" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF9" s="1" t="s">
         <v>40</v>
-      </c>
-      <c r="R9" s="1">
-        <v>0</v>
-      </c>
-      <c r="S9" s="1">
-        <v>160</v>
-      </c>
-      <c r="T9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U9" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="V9" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="W9" s="1">
-        <v>0</v>
-      </c>
-      <c r="X9" s="1">
-        <v>235</v>
-      </c>
-      <c r="Y9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z9" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA9" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE9" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AF9" s="1" t="s">
-        <v>15</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
@@ -1977,7 +1980,7 @@
         <v>123</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="AP9" s="1" t="s">
         <v>23</v>
@@ -1986,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>254</v>
+        <v>186</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
@@ -2036,16 +2039,16 @@
         <v>123</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="Q10" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="R10" s="1">
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>187</v>
+        <v>115</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>123</v>
@@ -2075,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>287</v>
+        <v>415</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
@@ -2111,16 +2114,16 @@
         <v>123</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>108</v>
+        <v>99</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>299</v>
+        <v>254</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
@@ -2164,7 +2167,7 @@
         <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>142</v>
+        <v>190</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>123</v>
@@ -2200,16 +2203,16 @@
         <v>123</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>20</v>
+        <v>211</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
@@ -2245,16 +2248,16 @@
         <v>123</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>117</v>
+        <v>108</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="AQ11" s="1">
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>303</v>
+        <v>299</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
@@ -2328,22 +2331,22 @@
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>247</v>
+        <v>271</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AB12" s="1">
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>84</v>
+        <v>284</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
@@ -2379,16 +2382,16 @@
         <v>123</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>35</v>
+        <v>117</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>21</v>
+        <v>40</v>
       </c>
       <c r="AQ12" s="1">
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>282</v>
+        <v>303</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2462,7 +2465,7 @@
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>291</v>
+        <v>297</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>123</v>
@@ -2492,7 +2495,7 @@
         <v>0</v>
       </c>
       <c r="AH13" s="1">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>123</v>
@@ -2513,150 +2516,284 @@
         <v>123</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>82</v>
+        <v>35</v>
       </c>
       <c r="AP13" s="1" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="AQ13" s="1">
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>422</v>
+        <v>442</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="G14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="I14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="J14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="L14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="N14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="O14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Q14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="S14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="T14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="V14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="W14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="X14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Y14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AA14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AC14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AD14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AF14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AG14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AH14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AI14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AK14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AM14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AN14" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO14" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="AP14" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AQ14" s="1">
+        <v>0</v>
+      </c>
+      <c r="AR14" s="1">
+        <v>422</v>
+      </c>
+    </row>
+    <row r="15" spans="1:44" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="B14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="C14" s="1">
-        <v>0</v>
-      </c>
-      <c r="D14" s="1">
+      <c r="B15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C15" s="1">
+        <v>0</v>
+      </c>
+      <c r="D15" s="1">
         <v>1369</v>
       </c>
-      <c r="E14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F14" s="1" t="s">
+      <c r="E15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="G14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="H14" s="1">
-        <v>0</v>
-      </c>
-      <c r="I14" s="1">
-        <v>2090</v>
-      </c>
-      <c r="J14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K14" s="1" t="s">
+      <c r="G15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="H15" s="1">
+        <v>0</v>
+      </c>
+      <c r="I15" s="1">
+        <v>2102</v>
+      </c>
+      <c r="J15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="L14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="M14" s="1">
-        <v>0</v>
-      </c>
-      <c r="N14" s="1">
-        <v>2557</v>
-      </c>
-      <c r="O14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P14" s="1" t="s">
+      <c r="L15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="M15" s="1">
+        <v>0</v>
+      </c>
+      <c r="N15" s="1">
+        <v>2605</v>
+      </c>
+      <c r="O15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="Q14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="R14" s="1">
-        <v>0</v>
-      </c>
-      <c r="S14" s="1">
-        <v>2043</v>
-      </c>
-      <c r="T14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U14" s="1" t="s">
+      <c r="Q15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="R15" s="1">
+        <v>0</v>
+      </c>
+      <c r="S15" s="1">
+        <v>2068</v>
+      </c>
+      <c r="T15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="V14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="W14" s="1">
-        <v>0</v>
-      </c>
-      <c r="X14" s="1">
-        <v>1990</v>
-      </c>
-      <c r="Y14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z14" s="1" t="s">
+      <c r="V15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="W15" s="1">
+        <v>0</v>
+      </c>
+      <c r="X15" s="1">
+        <v>2053</v>
+      </c>
+      <c r="Y15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="AA14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AB14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC14" s="1">
-        <v>1871</v>
-      </c>
-      <c r="AD14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE14" s="1" t="s">
+      <c r="AA15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC15" s="1">
+        <v>2193</v>
+      </c>
+      <c r="AD15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="AF14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AG14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH14" s="1">
-        <v>2051</v>
-      </c>
-      <c r="AI14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ14" s="1" t="s">
+      <c r="AF15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AG15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH15" s="1">
+        <v>2315</v>
+      </c>
+      <c r="AI15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="AK14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AL14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM14" s="1">
+      <c r="AK15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AL15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM15" s="1">
         <v>2691</v>
       </c>
-      <c r="AN14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO14" s="1" t="s">
+      <c r="AN15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO15" s="1" t="s">
         <v>118</v>
       </c>
-      <c r="AP14" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AQ14" s="1">
-        <v>0</v>
-      </c>
-      <c r="AR14" s="1">
-        <v>2739</v>
+      <c r="AP15" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AQ15" s="1">
+        <v>0</v>
+      </c>
+      <c r="AR15" s="1">
+        <v>2909</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 25
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9AE742CC-8446-46AF-88CC-051601248765}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4ABFCF89-94BE-4F14-8D7F-580675DB7926}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2592" yWindow="2028" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3288" yWindow="2724" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1116,46 +1116,46 @@
         <v>123</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>50</v>
+        <v>86</v>
       </c>
       <c r="V3" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="W3" s="1">
         <v>0</v>
       </c>
       <c r="X3" s="1">
-        <v>268</v>
+        <v>185</v>
       </c>
       <c r="Y3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>217</v>
+        <v>95</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE3" s="1" t="s">
-        <v>62</v>
+        <v>22</v>
       </c>
       <c r="AF3" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="AG3" s="1">
         <v>0</v>
       </c>
       <c r="AH3" s="1">
-        <v>124</v>
+        <v>281</v>
       </c>
       <c r="AI3" s="1" t="s">
         <v>123</v>
@@ -1190,31 +1190,31 @@
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>100</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
       </c>
       <c r="D4" s="1">
+        <v>171</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="G4" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="E4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>160</v>
+        <v>470</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
@@ -1250,37 +1250,37 @@
         <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>104</v>
+        <v>50</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>0</v>
+        <v>268</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>61</v>
+        <v>42</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>34</v>
+        <v>24</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>189</v>
+        <v>217</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>22</v>
+        <v>88</v>
       </c>
       <c r="AF4" s="1" t="s">
         <v>15</v>
@@ -1289,7 +1289,7 @@
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>281</v>
+        <v>220</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>123</v>
@@ -1324,31 +1324,31 @@
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>100</v>
+        <v>56</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
       </c>
       <c r="D5" s="1">
-        <v>171</v>
+        <v>114</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>121</v>
+        <v>47</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>470</v>
+        <v>103</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>123</v>
@@ -1369,61 +1369,61 @@
         <v>123</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>68</v>
+        <v>112</v>
       </c>
       <c r="Q5" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
+        <v>132</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="V5" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="R5" s="1">
-        <v>0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>0</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>118</v>
+        <v>0</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>79</v>
+        <v>61</v>
       </c>
       <c r="AA5" s="1" t="s">
-        <v>17</v>
+        <v>34</v>
       </c>
       <c r="AB5" s="1">
         <v>0</v>
       </c>
       <c r="AC5" s="1">
-        <v>170</v>
+        <v>189</v>
       </c>
       <c r="AD5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>97</v>
+        <v>43</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="AG5" s="1">
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>243</v>
+        <v>145</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
@@ -1473,16 +1473,16 @@
         <v>123</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>123</v>
@@ -1503,7 +1503,7 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>112</v>
+        <v>39</v>
       </c>
       <c r="Q6" s="1" t="s">
         <v>40</v>
@@ -1512,28 +1512,28 @@
         <v>0</v>
       </c>
       <c r="S6" s="1">
-        <v>132</v>
+        <v>160</v>
       </c>
       <c r="T6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>69</v>
+        <v>41</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>54</v>
+        <v>29</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>300</v>
+        <v>328</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="AA6" s="1" t="s">
         <v>17</v>
@@ -1542,13 +1542,13 @@
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>351</v>
+        <v>170</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="AF6" s="1" t="s">
         <v>15</v>
@@ -1557,7 +1557,7 @@
         <v>0</v>
       </c>
       <c r="AH6" s="1">
-        <v>220</v>
+        <v>210</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>123</v>
@@ -1607,16 +1607,16 @@
         <v>123</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>26</v>
+        <v>75</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H7" s="1">
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>241</v>
+        <v>0</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>123</v>
@@ -1637,61 +1637,61 @@
         <v>123</v>
       </c>
       <c r="P7" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
         <v>39</v>
       </c>
-      <c r="Q7" s="1" t="s">
+      <c r="T7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0</v>
+      </c>
+      <c r="X7" s="1">
+        <v>118</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA7" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB7" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC7" s="1">
+        <v>351</v>
+      </c>
+      <c r="AD7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE7" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF7" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="R7" s="1">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>160</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="W7" s="1">
-        <v>0</v>
-      </c>
-      <c r="X7" s="1">
-        <v>181</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z7" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC7" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE7" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AF7" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>145</v>
+        <v>0</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
@@ -1726,31 +1726,31 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>65</v>
+        <v>83</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>146</v>
+        <v>0</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>66</v>
+        <v>37</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>61</v>
+        <v>160</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
@@ -1786,22 +1786,22 @@
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>41</v>
+        <v>69</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>270</v>
+        <v>300</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>51</v>
+        <v>105</v>
       </c>
       <c r="AA8" s="1" t="s">
         <v>24</v>
@@ -1810,22 +1810,22 @@
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>32</v>
+        <v>115</v>
       </c>
       <c r="AF8" s="1" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>210</v>
+        <v>265</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
@@ -1860,10 +1860,10 @@
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
@@ -1875,16 +1875,16 @@
         <v>123</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>0</v>
+        <v>285</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
@@ -1920,46 +1920,46 @@
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>60</v>
+        <v>78</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="W9" s="1">
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>38</v>
+        <v>181</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>70</v>
+        <v>51</v>
       </c>
       <c r="AA9" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC9" s="1">
+        <v>20</v>
+      </c>
+      <c r="AD9" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE9" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF9" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AB9" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC9" s="1">
-        <v>84</v>
-      </c>
-      <c r="AD9" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF9" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>0</v>
+        <v>171</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -1989,21 +1989,21 @@
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>186</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>91</v>
+        <v>109</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>123</v>
@@ -2054,16 +2054,16 @@
         <v>123</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>113</v>
+        <v>60</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>54</v>
+        <v>13</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>138</v>
+        <v>38</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>123</v>
@@ -2084,16 +2084,16 @@
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>115</v>
+        <v>97</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>265</v>
+        <v>381</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
@@ -2123,21 +2123,21 @@
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>254</v>
+        <v>275</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>109</v>
+        <v>65</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>45</v>
+        <v>311</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
@@ -2188,16 +2188,16 @@
         <v>123</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>86</v>
+        <v>113</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>29</v>
+        <v>54</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>172</v>
+        <v>138</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>123</v>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="S12" s="1">
-        <v>308</v>
+        <v>360</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>123</v>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>345</v>
+        <v>509</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
@@ -2420,7 +2420,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>123</v>
@@ -2435,7 +2435,7 @@
         <v>0</v>
       </c>
       <c r="N13" s="1">
-        <v>406</v>
+        <v>504</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>123</v>
@@ -2510,7 +2510,7 @@
         <v>0</v>
       </c>
       <c r="AM13" s="1">
-        <v>361</v>
+        <v>381</v>
       </c>
       <c r="AN13" s="1" t="s">
         <v>123</v>
@@ -2659,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>422</v>
+        <v>479</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="1">
-        <v>1369</v>
+        <v>1608</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>123</v>
@@ -2688,7 +2688,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="1">
-        <v>2102</v>
+        <v>2148</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>123</v>
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="1">
-        <v>2605</v>
+        <v>2703</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>123</v>
@@ -2718,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="1">
-        <v>2068</v>
+        <v>2159</v>
       </c>
       <c r="T15" s="1" t="s">
         <v>123</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>2053</v>
+        <v>2124</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>123</v>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>2193</v>
+        <v>2204</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>123</v>
@@ -2763,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="1">
-        <v>2315</v>
+        <v>2500</v>
       </c>
       <c r="AI15" s="1" t="s">
         <v>123</v>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="AM15" s="1">
-        <v>2691</v>
+        <v>2875</v>
       </c>
       <c r="AN15" s="1" t="s">
         <v>123</v>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="AR15" s="1">
-        <v>2909</v>
+        <v>3101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 29
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1B1E294-73E3-48FB-A79F-FBEB3D50A0F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC36D3F-C665-4A8D-B124-D0174F83A081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3636" yWindow="3072" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1056,16 +1056,16 @@
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>46</v>
+        <v>25</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>456</v>
+        <v>0</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>123</v>
@@ -1161,45 +1161,45 @@
         <v>123</v>
       </c>
       <c r="AJ3" s="1" t="s">
-        <v>89</v>
+        <v>72</v>
       </c>
       <c r="AK3" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="AL3" s="1">
         <v>0</v>
       </c>
       <c r="AM3" s="1">
-        <v>0</v>
+        <v>401</v>
       </c>
       <c r="AN3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>361</v>
+        <v>323</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
       </c>
       <c r="D4" s="1">
-        <v>114</v>
+        <v>0</v>
       </c>
       <c r="E4" s="1" t="s">
         <v>123</v>
@@ -1235,99 +1235,99 @@
         <v>123</v>
       </c>
       <c r="P4" s="1" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="Q4" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R4" s="1">
+        <v>0</v>
+      </c>
+      <c r="S4" s="1">
+        <v>180</v>
+      </c>
+      <c r="T4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="V4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="W4" s="1">
+        <v>0</v>
+      </c>
+      <c r="X4" s="1">
+        <v>171</v>
+      </c>
+      <c r="Y4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z4" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="AA4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB4" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC4" s="1">
+        <v>170</v>
+      </c>
+      <c r="AD4" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE4" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="AF4" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="R4" s="1">
-        <v>0</v>
-      </c>
-      <c r="S4" s="1">
-        <v>417</v>
-      </c>
-      <c r="T4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U4" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="V4" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="W4" s="1">
-        <v>0</v>
-      </c>
-      <c r="X4" s="1">
-        <v>185</v>
-      </c>
-      <c r="Y4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z4" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="AA4" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="AB4" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC4" s="1">
-        <v>189</v>
-      </c>
-      <c r="AD4" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE4" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF4" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AG4" s="1">
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>0</v>
+        <v>432</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ4" s="1" t="s">
-        <v>53</v>
+        <v>89</v>
       </c>
       <c r="AK4" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="AL4" s="1">
         <v>0</v>
       </c>
       <c r="AM4" s="1">
-        <v>88</v>
+        <v>0</v>
       </c>
       <c r="AN4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>124</v>
+        <v>120</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>10</v>
+        <v>361</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>25</v>
+        <v>83</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -1339,16 +1339,16 @@
         <v>123</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H5" s="1">
         <v>0</v>
       </c>
       <c r="I5" s="1">
-        <v>103</v>
+        <v>61</v>
       </c>
       <c r="J5" s="1" t="s">
         <v>123</v>
@@ -1369,82 +1369,82 @@
         <v>123</v>
       </c>
       <c r="P5" s="1" t="s">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="Q5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="R5" s="1">
+        <v>0</v>
+      </c>
+      <c r="S5" s="1">
+        <v>137</v>
+      </c>
+      <c r="T5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U5" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V5" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W5" s="1">
+        <v>0</v>
+      </c>
+      <c r="X5" s="1">
+        <v>352</v>
+      </c>
+      <c r="Y5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z5" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AB5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>95</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="AF5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="R5" s="1">
-        <v>0</v>
-      </c>
-      <c r="S5" s="1">
-        <v>180</v>
-      </c>
-      <c r="T5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U5" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="V5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="W5" s="1">
-        <v>0</v>
-      </c>
-      <c r="X5" s="1">
-        <v>328</v>
-      </c>
-      <c r="Y5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z5" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA5" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="AB5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="1">
-        <v>170</v>
-      </c>
-      <c r="AD5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE5" s="1" t="s">
-        <v>62</v>
-      </c>
-      <c r="AF5" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="AG5" s="1">
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>97</v>
+        <v>123</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>90</v>
+        <v>124</v>
       </c>
       <c r="AP5" s="1" t="s">
         <v>29</v>
@@ -1453,15 +1453,15 @@
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>36</v>
+        <v>91</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -1473,16 +1473,16 @@
         <v>123</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>66</v>
+        <v>75</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>40</v>
+        <v>24</v>
       </c>
       <c r="H6" s="1">
         <v>0</v>
       </c>
       <c r="I6" s="1">
-        <v>61</v>
+        <v>0</v>
       </c>
       <c r="J6" s="1" t="s">
         <v>123</v>
@@ -1503,96 +1503,96 @@
         <v>123</v>
       </c>
       <c r="P6" s="1" t="s">
-        <v>49</v>
+        <v>112</v>
       </c>
       <c r="Q6" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R6" s="1">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1">
+        <v>160</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="W6" s="1">
+        <v>0</v>
+      </c>
+      <c r="X6" s="1">
+        <v>455</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="R6" s="1">
-        <v>0</v>
-      </c>
-      <c r="S6" s="1">
-        <v>137</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="V6" s="1" t="s">
+      <c r="AB6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC6" s="1">
+        <v>423</v>
+      </c>
+      <c r="AD6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE6" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF6" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="AG6" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH6" s="1">
+        <v>171</v>
+      </c>
+      <c r="AI6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ6" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="AK6" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="W6" s="1">
-        <v>0</v>
-      </c>
-      <c r="X6" s="1">
-        <v>171</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AB6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC6" s="1">
-        <v>95</v>
-      </c>
-      <c r="AD6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE6" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="AF6" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG6" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH6" s="1">
-        <v>220</v>
-      </c>
-      <c r="AI6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ6" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="AK6" s="1" t="s">
-        <v>34</v>
-      </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>392</v>
+        <v>97</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>293</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>83</v>
+        <v>109</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>24</v>
@@ -1601,88 +1601,88 @@
         <v>0</v>
       </c>
       <c r="D7" s="1">
-        <v>0</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>75</v>
+        <v>26</v>
       </c>
       <c r="G7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>285</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>313</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
+        <v>187</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0</v>
+      </c>
+      <c r="X7" s="1">
+        <v>59</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AA7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H7" s="1">
-        <v>0</v>
-      </c>
-      <c r="I7" s="1">
-        <v>0</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-      <c r="N7" s="1">
-        <v>269</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="R7" s="1">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>160</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="W7" s="1">
-        <v>0</v>
-      </c>
-      <c r="X7" s="1">
-        <v>300</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="AB7" s="1">
         <v>0</v>
       </c>
       <c r="AC7" s="1">
-        <v>423</v>
+        <v>0</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>43</v>
+        <v>88</v>
       </c>
       <c r="AF7" s="1" t="s">
         <v>15</v>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>145</v>
+        <v>220</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
@@ -1712,111 +1712,111 @@
         <v>123</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>117</v>
+        <v>45</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="AQ7" s="1">
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>369</v>
+        <v>293</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>0</v>
+        <v>237</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>26</v>
+        <v>14</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>285</v>
+        <v>69</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>16</v>
+        <v>102</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="M8" s="1">
         <v>0</v>
       </c>
       <c r="N8" s="1">
-        <v>392</v>
+        <v>292</v>
       </c>
       <c r="O8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>68</v>
+        <v>94</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>39</v>
+        <v>94</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>50</v>
+        <v>113</v>
       </c>
       <c r="V8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0</v>
+      </c>
+      <c r="X8" s="1">
+        <v>138</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="AA8" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W8" s="1">
-        <v>0</v>
-      </c>
-      <c r="X8" s="1">
-        <v>268</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>0</v>
+        <v>332</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE8" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="AF8" s="1" t="s">
         <v>15</v>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>210</v>
+        <v>145</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
@@ -1846,30 +1846,30 @@
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>73</v>
+        <v>117</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>300</v>
+        <v>369</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>109</v>
+        <v>119</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>45</v>
+        <v>497</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>123</v>
@@ -1884,52 +1884,52 @@
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>160</v>
+        <v>204</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>58</v>
+        <v>67</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="M9" s="1">
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>280</v>
+        <v>227</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>28</v>
+        <v>77</v>
       </c>
       <c r="Q9" s="1" t="s">
-        <v>29</v>
+        <v>15</v>
       </c>
       <c r="R9" s="1">
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>187</v>
+        <v>240</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>60</v>
+        <v>19</v>
       </c>
       <c r="V9" s="1" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="W9" s="1">
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>59</v>
+        <v>271</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
@@ -1950,16 +1950,16 @@
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>97</v>
+        <v>32</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>381</v>
+        <v>210</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
@@ -1980,7 +1980,7 @@
         <v>123</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>99</v>
+        <v>73</v>
       </c>
       <c r="AP9" s="1" t="s">
         <v>23</v>
@@ -1989,57 +1989,57 @@
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>275</v>
+        <v>300</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>100</v>
+        <v>65</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>237</v>
+        <v>388</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>14</v>
+        <v>92</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H10" s="1">
         <v>0</v>
       </c>
       <c r="I10" s="1">
-        <v>69</v>
+        <v>446</v>
       </c>
       <c r="J10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>102</v>
+        <v>16</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="M10" s="1">
         <v>0</v>
       </c>
       <c r="N10" s="1">
-        <v>219</v>
+        <v>392</v>
       </c>
       <c r="O10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P10" s="1" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="Q10" s="1" t="s">
         <v>15</v>
@@ -2048,22 +2048,22 @@
         <v>0</v>
       </c>
       <c r="S10" s="1">
-        <v>240</v>
+        <v>115</v>
       </c>
       <c r="T10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U10" s="1" t="s">
-        <v>113</v>
+        <v>95</v>
       </c>
       <c r="V10" s="1" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="W10" s="1">
         <v>0</v>
       </c>
       <c r="X10" s="1">
-        <v>138</v>
+        <v>297</v>
       </c>
       <c r="Y10" s="1" t="s">
         <v>123</v>
@@ -2078,22 +2078,22 @@
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>415</v>
+        <v>432</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>106</v>
+        <v>97</v>
       </c>
       <c r="AF10" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="AG10" s="1">
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>392</v>
+        <v>381</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
@@ -2114,21 +2114,21 @@
         <v>123</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>108</v>
+        <v>35</v>
       </c>
       <c r="AP10" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>426</v>
+        <v>452</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>56</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>29</v>
@@ -2137,67 +2137,67 @@
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>311</v>
+        <v>258</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>92</v>
+        <v>47</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
       </c>
       <c r="I11" s="1">
+        <v>120</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M11" s="1">
+        <v>0</v>
+      </c>
+      <c r="N11" s="1">
+        <v>376</v>
+      </c>
+      <c r="O11" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P11" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="Q11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="R11" s="1">
+        <v>0</v>
+      </c>
+      <c r="S11" s="1">
         <v>446</v>
       </c>
-      <c r="J11" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K11" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="L11" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="M11" s="1">
-        <v>0</v>
-      </c>
-      <c r="N11" s="1">
-        <v>190</v>
-      </c>
-      <c r="O11" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P11" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q11" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="R11" s="1">
-        <v>0</v>
-      </c>
-      <c r="S11" s="1">
-        <v>115</v>
-      </c>
       <c r="T11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>19</v>
+        <v>78</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>15</v>
+        <v>24</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>271</v>
+        <v>205</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>123</v>
@@ -2212,7 +2212,7 @@
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>211</v>
+        <v>288</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
@@ -2227,7 +2227,7 @@
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>379</v>
+        <v>451</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
@@ -2248,30 +2248,30 @@
         <v>123</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AQ11" s="1">
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>442</v>
+        <v>275</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>119</v>
+        <v>46</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>13</v>
+        <v>34</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>497</v>
+        <v>550</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>123</v>
@@ -2292,16 +2292,16 @@
         <v>123</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>93</v>
+        <v>38</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>223</v>
+        <v>382</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>123</v>
@@ -2322,31 +2322,31 @@
         <v>123</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>95</v>
+        <v>86</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>15</v>
+        <v>29</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AB12" s="1">
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>284</v>
+        <v>209</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
@@ -2367,31 +2367,31 @@
         <v>123</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>72</v>
+        <v>33</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>381</v>
+        <v>469</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>82</v>
+        <v>108</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>23</v>
+        <v>13</v>
       </c>
       <c r="AQ12" s="1">
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>479</v>
+        <v>426</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
@@ -2420,7 +2420,7 @@
         <v>0</v>
       </c>
       <c r="I13" s="1">
-        <v>276</v>
+        <v>286</v>
       </c>
       <c r="J13" s="1" t="s">
         <v>123</v>
@@ -2441,31 +2441,31 @@
         <v>123</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>94</v>
+        <v>68</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="R13" s="1">
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U13" s="1" t="s">
-        <v>78</v>
+        <v>41</v>
       </c>
       <c r="V13" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="W13" s="1">
         <v>0</v>
       </c>
       <c r="X13" s="1">
-        <v>205</v>
+        <v>430</v>
       </c>
       <c r="Y13" s="1" t="s">
         <v>123</v>
@@ -2495,7 +2495,7 @@
         <v>0</v>
       </c>
       <c r="AH13" s="1">
-        <v>56</v>
+        <v>127</v>
       </c>
       <c r="AI13" s="1" t="s">
         <v>123</v>
@@ -2516,16 +2516,16 @@
         <v>123</v>
       </c>
       <c r="AO13" s="1" t="s">
-        <v>55</v>
+        <v>82</v>
       </c>
       <c r="AP13" s="1" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="AQ13" s="1">
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>238</v>
+        <v>479</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2659,7 +2659,7 @@
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>260</v>
+        <v>268</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="1">
-        <v>1676</v>
+        <v>1991</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>123</v>
@@ -2688,7 +2688,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="1">
-        <v>2447</v>
+        <v>2518</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>123</v>
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="1">
-        <v>2882</v>
+        <v>3291</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>123</v>
@@ -2718,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="1">
-        <v>2281</v>
+        <v>2364</v>
       </c>
       <c r="T15" s="1" t="s">
         <v>123</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>2222</v>
+        <v>2664</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>123</v>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>2427</v>
+        <v>2589</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>123</v>
@@ -2763,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="1">
-        <v>2581</v>
+        <v>2764</v>
       </c>
       <c r="AI15" s="1" t="s">
         <v>123</v>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="AM15" s="1">
-        <v>3217</v>
+        <v>3349</v>
       </c>
       <c r="AN15" s="1" t="s">
         <v>123</v>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="AR15" s="1">
-        <v>3453</v>
+        <v>3556</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 30
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1AC36D3F-C665-4A8D-B124-D0174F83A081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD004E8-E96E-4BB9-AE3F-55985E91B31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3636" yWindow="3072" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1131,16 +1131,16 @@
         <v>123</v>
       </c>
       <c r="Z3" s="1" t="s">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="AA3" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AB3" s="1">
         <v>0</v>
       </c>
       <c r="AC3" s="1">
-        <v>319</v>
+        <v>109</v>
       </c>
       <c r="AD3" s="1" t="s">
         <v>123</v>
@@ -1176,16 +1176,16 @@
         <v>123</v>
       </c>
       <c r="AO3" s="1" t="s">
-        <v>55</v>
+        <v>120</v>
       </c>
       <c r="AP3" s="1" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>323</v>
+        <v>361</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
@@ -1265,16 +1265,16 @@
         <v>123</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>79</v>
+        <v>42</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>170</v>
+        <v>319</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
@@ -1310,16 +1310,16 @@
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>361</v>
+        <v>10</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
@@ -1384,67 +1384,67 @@
         <v>123</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>69</v>
+        <v>50</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>54</v>
+        <v>21</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>352</v>
+        <v>455</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z5" s="1" t="s">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="AA5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="AB5" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC5" s="1">
+        <v>332</v>
+      </c>
+      <c r="AD5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE5" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF5" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AB5" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC5" s="1">
-        <v>95</v>
-      </c>
-      <c r="AD5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE5" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="AF5" s="1" t="s">
-        <v>40</v>
-      </c>
       <c r="AG5" s="1">
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>0</v>
+        <v>189</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>123</v>
+        <v>469</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>124</v>
+        <v>90</v>
       </c>
       <c r="AP5" s="1" t="s">
         <v>29</v>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
@@ -1488,16 +1488,16 @@
         <v>123</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>48</v>
+        <v>93</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="M6" s="1">
         <v>0</v>
       </c>
       <c r="N6" s="1">
-        <v>270</v>
+        <v>313</v>
       </c>
       <c r="O6" s="1" t="s">
         <v>123</v>
@@ -1518,22 +1518,22 @@
         <v>123</v>
       </c>
       <c r="U6" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V6" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="W6" s="1">
         <v>0</v>
       </c>
       <c r="X6" s="1">
-        <v>455</v>
+        <v>59</v>
       </c>
       <c r="Y6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z6" s="1" t="s">
-        <v>96</v>
+        <v>79</v>
       </c>
       <c r="AA6" s="1" t="s">
         <v>17</v>
@@ -1542,22 +1542,22 @@
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>423</v>
+        <v>170</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE6" s="1" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="AF6" s="1" t="s">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="AG6" s="1">
         <v>0</v>
       </c>
       <c r="AH6" s="1">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="AI6" s="1" t="s">
         <v>123</v>
@@ -1578,16 +1578,16 @@
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>90</v>
+        <v>45</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>0</v>
+        <v>293</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
@@ -1616,28 +1616,28 @@
         <v>0</v>
       </c>
       <c r="I7" s="1">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="J7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>93</v>
+        <v>48</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="M7" s="1">
         <v>0</v>
       </c>
       <c r="N7" s="1">
-        <v>313</v>
+        <v>270</v>
       </c>
       <c r="O7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P7" s="1" t="s">
-        <v>28</v>
+        <v>68</v>
       </c>
       <c r="Q7" s="1" t="s">
         <v>29</v>
@@ -1646,111 +1646,111 @@
         <v>0</v>
       </c>
       <c r="S7" s="1">
-        <v>187</v>
+        <v>66</v>
       </c>
       <c r="T7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U7" s="1" t="s">
-        <v>60</v>
+        <v>113</v>
       </c>
       <c r="V7" s="1" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="W7" s="1">
         <v>0</v>
       </c>
       <c r="X7" s="1">
-        <v>59</v>
+        <v>138</v>
       </c>
       <c r="Y7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z7" s="1" t="s">
-        <v>105</v>
+        <v>96</v>
       </c>
       <c r="AA7" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="AB7" s="1">
         <v>0</v>
       </c>
       <c r="AC7" s="1">
-        <v>0</v>
+        <v>423</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE7" s="1" t="s">
-        <v>88</v>
+        <v>97</v>
       </c>
       <c r="AF7" s="1" t="s">
-        <v>15</v>
+        <v>23</v>
       </c>
       <c r="AG7" s="1">
         <v>0</v>
       </c>
       <c r="AH7" s="1">
-        <v>220</v>
+        <v>553</v>
       </c>
       <c r="AI7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>63</v>
+        <v>122</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>253</v>
+        <v>539</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO7" s="1" t="s">
-        <v>45</v>
+        <v>117</v>
       </c>
       <c r="AP7" s="1" t="s">
-        <v>17</v>
+        <v>40</v>
       </c>
       <c r="AQ7" s="1">
         <v>0</v>
       </c>
       <c r="AR7" s="1">
-        <v>293</v>
+        <v>369</v>
       </c>
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>100</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="C8" s="1">
         <v>0</v>
       </c>
       <c r="D8" s="1">
-        <v>237</v>
+        <v>550</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>14</v>
+        <v>47</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="H8" s="1">
         <v>0</v>
       </c>
       <c r="I8" s="1">
-        <v>69</v>
+        <v>120</v>
       </c>
       <c r="J8" s="1" t="s">
         <v>123</v>
@@ -1771,46 +1771,46 @@
         <v>123</v>
       </c>
       <c r="P8" s="1" t="s">
-        <v>94</v>
+        <v>59</v>
       </c>
       <c r="Q8" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="R8" s="1">
         <v>0</v>
       </c>
       <c r="S8" s="1">
-        <v>94</v>
+        <v>446</v>
       </c>
       <c r="T8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U8" s="1" t="s">
-        <v>113</v>
+        <v>19</v>
       </c>
       <c r="V8" s="1" t="s">
-        <v>54</v>
+        <v>15</v>
       </c>
       <c r="W8" s="1">
         <v>0</v>
       </c>
       <c r="X8" s="1">
-        <v>138</v>
+        <v>334</v>
       </c>
       <c r="Y8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z8" s="1" t="s">
-        <v>20</v>
+        <v>105</v>
       </c>
       <c r="AA8" s="1" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="AB8" s="1">
         <v>0</v>
       </c>
       <c r="AC8" s="1">
-        <v>332</v>
+        <v>0</v>
       </c>
       <c r="AD8" s="1" t="s">
         <v>123</v>
@@ -1825,87 +1825,87 @@
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>145</v>
+        <v>348</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>81</v>
+        <v>63</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>54</v>
+        <v>24</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>166</v>
+        <v>253</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>117</v>
+        <v>35</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>40</v>
+        <v>21</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>369</v>
+        <v>452</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>119</v>
+        <v>100</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>497</v>
+        <v>237</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>37</v>
+        <v>14</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>204</v>
+        <v>69</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>67</v>
+        <v>38</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="M9" s="1">
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>227</v>
+        <v>382</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>77</v>
+        <v>18</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>15</v>
@@ -1914,13 +1914,13 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>240</v>
+        <v>177</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>15</v>
@@ -1929,52 +1929,52 @@
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>271</v>
+        <v>297</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>51</v>
+        <v>61</v>
       </c>
       <c r="AA9" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="AB9" s="1">
         <v>0</v>
       </c>
       <c r="AC9" s="1">
-        <v>24</v>
+        <v>209</v>
       </c>
       <c r="AD9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>15</v>
+        <v>34</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>210</v>
+        <v>451</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>44</v>
+        <v>81</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>24</v>
+        <v>54</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
       </c>
       <c r="AM9" s="1">
-        <v>307</v>
+        <v>166</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>123</v>
@@ -1989,146 +1989,146 @@
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>300</v>
+        <v>358</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>65</v>
+        <v>119</v>
       </c>
       <c r="B10" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C10" s="1">
+        <v>0</v>
+      </c>
+      <c r="D10" s="1">
+        <v>497</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>204</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M10" s="1">
+        <v>0</v>
+      </c>
+      <c r="N10" s="1">
+        <v>227</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q10" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
-        <v>388</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>92</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>446</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="L10" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="M10" s="1">
-        <v>0</v>
-      </c>
-      <c r="N10" s="1">
-        <v>392</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="Q10" s="1" t="s">
+      <c r="R10" s="1">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
+        <v>187</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W10" s="1">
+        <v>0</v>
+      </c>
+      <c r="X10" s="1">
+        <v>352</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z10" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC10" s="1">
+        <v>24</v>
+      </c>
+      <c r="AD10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE10" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="AF10" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="R10" s="1">
-        <v>0</v>
-      </c>
-      <c r="S10" s="1">
-        <v>115</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W10" s="1">
-        <v>0</v>
-      </c>
-      <c r="X10" s="1">
-        <v>297</v>
-      </c>
-      <c r="Y10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z10" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="AA10" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="AB10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC10" s="1">
-        <v>432</v>
-      </c>
-      <c r="AD10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE10" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="AF10" s="1" t="s">
+      <c r="AG10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH10" s="1">
+        <v>267</v>
+      </c>
+      <c r="AI10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="AK10" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL10" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM10" s="1">
+        <v>307</v>
+      </c>
+      <c r="AN10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO10" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="AP10" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="AG10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH10" s="1">
-        <v>381</v>
-      </c>
-      <c r="AI10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ10" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="AK10" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="AL10" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM10" s="1">
-        <v>494</v>
-      </c>
-      <c r="AN10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO10" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="AP10" s="1" t="s">
-        <v>21</v>
-      </c>
       <c r="AQ10" s="1">
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>452</v>
+        <v>335</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>56</v>
+        <v>65</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>29</v>
@@ -2137,52 +2137,52 @@
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>258</v>
+        <v>388</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>47</v>
+        <v>92</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H11" s="1">
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>120</v>
+        <v>446</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>58</v>
+        <v>16</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>54</v>
+        <v>17</v>
       </c>
       <c r="M11" s="1">
         <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>376</v>
+        <v>392</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P11" s="1" t="s">
-        <v>59</v>
+        <v>94</v>
       </c>
       <c r="Q11" s="1" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="R11" s="1">
         <v>0</v>
       </c>
       <c r="S11" s="1">
-        <v>446</v>
+        <v>94</v>
       </c>
       <c r="T11" s="1" t="s">
         <v>123</v>
@@ -2203,7 +2203,7 @@
         <v>123</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="AA11" s="1" t="s">
         <v>21</v>
@@ -2212,66 +2212,66 @@
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>288</v>
+        <v>432</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>80</v>
+        <v>32</v>
       </c>
       <c r="AF11" s="1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="AG11" s="1">
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>451</v>
+        <v>241</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>122</v>
+        <v>53</v>
       </c>
       <c r="AK11" s="1" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="AL11" s="1">
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>509</v>
+        <v>123</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>99</v>
+        <v>55</v>
       </c>
       <c r="AP11" s="1" t="s">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="AQ11" s="1">
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>275</v>
+        <v>323</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>46</v>
+        <v>56</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>550</v>
+        <v>258</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>123</v>
@@ -2292,31 +2292,31 @@
         <v>123</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>38</v>
+        <v>58</v>
       </c>
       <c r="L12" s="1" t="s">
-        <v>34</v>
+        <v>54</v>
       </c>
       <c r="M12" s="1">
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>382</v>
+        <v>376</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="R12" s="1">
         <v>0</v>
       </c>
       <c r="S12" s="1">
-        <v>360</v>
+        <v>245</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>123</v>
@@ -2337,16 +2337,16 @@
         <v>123</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>61</v>
+        <v>87</v>
       </c>
       <c r="AA12" s="1" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="AB12" s="1">
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>209</v>
+        <v>288</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
@@ -2367,16 +2367,16 @@
         <v>123</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>33</v>
+        <v>116</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>34</v>
+        <v>13</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>469</v>
+        <v>494</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
@@ -2435,22 +2435,22 @@
         <v>0</v>
       </c>
       <c r="N13" s="1">
-        <v>504</v>
+        <v>517</v>
       </c>
       <c r="O13" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P13" s="1" t="s">
-        <v>68</v>
+        <v>85</v>
       </c>
       <c r="Q13" s="1" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="R13" s="1">
         <v>0</v>
       </c>
       <c r="S13" s="1">
-        <v>66</v>
+        <v>380</v>
       </c>
       <c r="T13" s="1" t="s">
         <v>123</v>
@@ -2525,7 +2525,7 @@
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>479</v>
+        <v>515</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2688,7 +2688,7 @@
         <v>0</v>
       </c>
       <c r="I15" s="1">
-        <v>2518</v>
+        <v>2520</v>
       </c>
       <c r="J15" s="1" t="s">
         <v>123</v>
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="1">
-        <v>3291</v>
+        <v>3304</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>123</v>
@@ -2718,7 +2718,7 @@
         <v>0</v>
       </c>
       <c r="S15" s="1">
-        <v>2364</v>
+        <v>2451</v>
       </c>
       <c r="T15" s="1" t="s">
         <v>123</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>2664</v>
+        <v>2727</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>123</v>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>2589</v>
+        <v>2603</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>123</v>
@@ -2763,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="1">
-        <v>2764</v>
+        <v>3235</v>
       </c>
       <c r="AI15" s="1" t="s">
         <v>123</v>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="AM15" s="1">
-        <v>3349</v>
+        <v>3379</v>
       </c>
       <c r="AN15" s="1" t="s">
         <v>123</v>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="AR15" s="1">
-        <v>3556</v>
+        <v>3710</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 31
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ipl26\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0FD004E8-E96E-4BB9-AE3F-55985E91B31E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17DE10C5-4E27-47A5-B2DD-EC39CB49B940}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="732" yWindow="732" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2688" yWindow="2688" windowWidth="17280" windowHeight="8880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Teams" sheetId="1" r:id="rId1"/>
@@ -1056,7 +1056,7 @@
     </row>
     <row r="3" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>25</v>
+        <v>119</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>13</v>
@@ -1065,135 +1065,135 @@
         <v>0</v>
       </c>
       <c r="D3" s="1">
-        <v>0</v>
+        <v>552</v>
       </c>
       <c r="E3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>110</v>
+        <v>101</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>40</v>
+        <v>13</v>
       </c>
       <c r="H3" s="1">
         <v>0</v>
       </c>
       <c r="I3" s="1">
-        <v>498</v>
+        <v>34</v>
       </c>
       <c r="J3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>111</v>
+        <v>76</v>
       </c>
       <c r="L3" s="1" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="M3" s="1">
         <v>0</v>
       </c>
       <c r="N3" s="1">
-        <v>535</v>
+        <v>0</v>
       </c>
       <c r="O3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P3" s="1" t="s">
-        <v>103</v>
+        <v>59</v>
       </c>
       <c r="Q3" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="R3" s="1">
         <v>0</v>
       </c>
       <c r="S3" s="1">
-        <v>379</v>
+        <v>446</v>
       </c>
       <c r="T3" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U3" s="1" t="s">
-        <v>104</v>
+        <v>78</v>
       </c>
       <c r="V3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="W3" s="1">
+        <v>0</v>
+      </c>
+      <c r="X3" s="1">
+        <v>213</v>
+      </c>
+      <c r="Y3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z3" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="AA3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AB3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC3" s="1">
+        <v>376</v>
+      </c>
+      <c r="AD3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE3" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="AF3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AG3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH3" s="1">
+        <v>360</v>
+      </c>
+      <c r="AI3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="AK3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AL3" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM3" s="1">
+        <v>256</v>
+      </c>
+      <c r="AN3" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO3" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="AP3" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="W3" s="1">
-        <v>0</v>
-      </c>
-      <c r="X3" s="1">
-        <v>0</v>
-      </c>
-      <c r="Y3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z3" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="AA3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="AB3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC3" s="1">
-        <v>109</v>
-      </c>
-      <c r="AD3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="AF3" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="AG3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="1">
-        <v>281</v>
-      </c>
-      <c r="AI3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ3" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="AK3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="AL3" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM3" s="1">
-        <v>401</v>
-      </c>
-      <c r="AN3" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO3" s="1" t="s">
-        <v>120</v>
-      </c>
-      <c r="AP3" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="AQ3" s="1">
         <v>0</v>
       </c>
       <c r="AR3" s="1">
-        <v>361</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>36</v>
+        <v>25</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C4" s="1">
         <v>0</v>
@@ -1205,25 +1205,25 @@
         <v>123</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>13</v>
+        <v>24</v>
       </c>
       <c r="H4" s="1">
         <v>0</v>
       </c>
       <c r="I4" s="1">
-        <v>34</v>
+        <v>0</v>
       </c>
       <c r="J4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>21</v>
+        <v>29</v>
       </c>
       <c r="M4" s="1">
         <v>0</v>
@@ -1250,46 +1250,46 @@
         <v>123</v>
       </c>
       <c r="U4" s="1" t="s">
-        <v>30</v>
+        <v>104</v>
       </c>
       <c r="V4" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="W4" s="1">
         <v>0</v>
       </c>
       <c r="X4" s="1">
-        <v>171</v>
+        <v>0</v>
       </c>
       <c r="Y4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z4" s="1" t="s">
-        <v>42</v>
+        <v>114</v>
       </c>
       <c r="AA4" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="AB4" s="1">
         <v>0</v>
       </c>
       <c r="AC4" s="1">
-        <v>319</v>
+        <v>364</v>
       </c>
       <c r="AD4" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE4" s="1" t="s">
-        <v>106</v>
+        <v>22</v>
       </c>
       <c r="AF4" s="1" t="s">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="AG4" s="1">
         <v>0</v>
       </c>
       <c r="AH4" s="1">
-        <v>432</v>
+        <v>281</v>
       </c>
       <c r="AI4" s="1" t="s">
         <v>123</v>
@@ -1310,24 +1310,24 @@
         <v>123</v>
       </c>
       <c r="AO4" s="1" t="s">
-        <v>124</v>
+        <v>45</v>
       </c>
       <c r="AP4" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="AQ4" s="1">
         <v>0</v>
       </c>
       <c r="AR4" s="1">
-        <v>10</v>
+        <v>293</v>
       </c>
     </row>
     <row r="5" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>83</v>
+        <v>36</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="C5" s="1">
         <v>0</v>
@@ -1339,61 +1339,61 @@
         <v>123</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>66</v>
+        <v>14</v>
       </c>
       <c r="G5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H5" s="1">
+        <v>0</v>
+      </c>
+      <c r="I5" s="1">
+        <v>69</v>
+      </c>
+      <c r="J5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K5" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="L5" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="M5" s="1">
+        <v>0</v>
+      </c>
+      <c r="N5" s="1">
+        <v>270</v>
+      </c>
+      <c r="O5" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P5" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="Q5" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1">
-        <v>61</v>
-      </c>
-      <c r="J5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K5" s="1" t="s">
-        <v>84</v>
-      </c>
-      <c r="L5" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="M5" s="1">
-        <v>0</v>
-      </c>
-      <c r="N5" s="1">
-        <v>0</v>
-      </c>
-      <c r="O5" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P5" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q5" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="R5" s="1">
         <v>0</v>
       </c>
       <c r="S5" s="1">
-        <v>137</v>
+        <v>160</v>
       </c>
       <c r="T5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U5" s="1" t="s">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="V5" s="1" t="s">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="W5" s="1">
         <v>0</v>
       </c>
       <c r="X5" s="1">
-        <v>455</v>
+        <v>71</v>
       </c>
       <c r="Y5" s="1" t="s">
         <v>123</v>
@@ -1414,54 +1414,54 @@
         <v>123</v>
       </c>
       <c r="AE5" s="1" t="s">
-        <v>62</v>
+        <v>106</v>
       </c>
       <c r="AF5" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="AG5" s="1">
         <v>0</v>
       </c>
       <c r="AH5" s="1">
-        <v>189</v>
+        <v>432</v>
       </c>
       <c r="AI5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ5" s="1" t="s">
-        <v>33</v>
+        <v>98</v>
       </c>
       <c r="AK5" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="AL5" s="1">
         <v>0</v>
       </c>
       <c r="AM5" s="1">
-        <v>469</v>
+        <v>97</v>
       </c>
       <c r="AN5" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO5" s="1" t="s">
-        <v>90</v>
+        <v>108</v>
       </c>
       <c r="AP5" s="1" t="s">
-        <v>29</v>
+        <v>13</v>
       </c>
       <c r="AQ5" s="1">
         <v>0</v>
       </c>
       <c r="AR5" s="1">
-        <v>0</v>
+        <v>705</v>
       </c>
     </row>
     <row r="6" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>91</v>
+        <v>83</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="1">
         <v>0</v>
@@ -1473,76 +1473,76 @@
         <v>123</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>75</v>
+        <v>47</v>
       </c>
       <c r="G6" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="H6" s="1">
+        <v>0</v>
+      </c>
+      <c r="I6" s="1">
+        <v>120</v>
+      </c>
+      <c r="J6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K6" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="L6" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" s="1">
+        <v>0</v>
+      </c>
+      <c r="N6" s="1">
+        <v>618</v>
+      </c>
+      <c r="O6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="Q6" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R6" s="1">
+        <v>0</v>
+      </c>
+      <c r="S6" s="1">
+        <v>187</v>
+      </c>
+      <c r="T6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U6" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="V6" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W6" s="1">
+        <v>0</v>
+      </c>
+      <c r="X6" s="1">
+        <v>138</v>
+      </c>
+      <c r="Y6" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z6" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="AA6" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="H6" s="1">
-        <v>0</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K6" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="L6" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M6" s="1">
-        <v>0</v>
-      </c>
-      <c r="N6" s="1">
-        <v>313</v>
-      </c>
-      <c r="O6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P6" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="Q6" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="R6" s="1">
-        <v>0</v>
-      </c>
-      <c r="S6" s="1">
-        <v>160</v>
-      </c>
-      <c r="T6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U6" s="1" t="s">
-        <v>60</v>
-      </c>
-      <c r="V6" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="W6" s="1">
-        <v>0</v>
-      </c>
-      <c r="X6" s="1">
-        <v>59</v>
-      </c>
-      <c r="Y6" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z6" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="AA6" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="AB6" s="1">
         <v>0</v>
       </c>
       <c r="AC6" s="1">
-        <v>170</v>
+        <v>0</v>
       </c>
       <c r="AD6" s="1" t="s">
         <v>123</v>
@@ -1563,120 +1563,120 @@
         <v>123</v>
       </c>
       <c r="AJ6" s="1" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="AK6" s="1" t="s">
-        <v>17</v>
+        <v>54</v>
       </c>
       <c r="AL6" s="1">
         <v>0</v>
       </c>
       <c r="AM6" s="1">
-        <v>97</v>
+        <v>166</v>
       </c>
       <c r="AN6" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO6" s="1" t="s">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="AP6" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="AQ6" s="1">
         <v>0</v>
       </c>
       <c r="AR6" s="1">
-        <v>293</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>109</v>
+        <v>91</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H7" s="1">
+        <v>0</v>
+      </c>
+      <c r="I7" s="1">
+        <v>446</v>
+      </c>
+      <c r="J7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="L7" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="M7" s="1">
+        <v>0</v>
+      </c>
+      <c r="N7" s="1">
+        <v>382</v>
+      </c>
+      <c r="O7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P7" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="Q7" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="R7" s="1">
+        <v>0</v>
+      </c>
+      <c r="S7" s="1">
+        <v>380</v>
+      </c>
+      <c r="T7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U7" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="V7" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="W7" s="1">
+        <v>0</v>
+      </c>
+      <c r="X7" s="1">
+        <v>430</v>
+      </c>
+      <c r="Y7" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="AA7" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C7" s="1">
-        <v>0</v>
-      </c>
-      <c r="D7" s="1">
-        <v>45</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="H7" s="1">
-        <v>0</v>
-      </c>
-      <c r="I7" s="1">
-        <v>287</v>
-      </c>
-      <c r="J7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K7" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="L7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-      <c r="N7" s="1">
-        <v>270</v>
-      </c>
-      <c r="O7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P7" s="1" t="s">
-        <v>68</v>
-      </c>
-      <c r="Q7" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="R7" s="1">
-        <v>0</v>
-      </c>
-      <c r="S7" s="1">
-        <v>66</v>
-      </c>
-      <c r="T7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U7" s="1" t="s">
-        <v>113</v>
-      </c>
-      <c r="V7" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="W7" s="1">
-        <v>0</v>
-      </c>
-      <c r="X7" s="1">
-        <v>138</v>
-      </c>
-      <c r="Y7" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z7" s="1" t="s">
-        <v>96</v>
-      </c>
-      <c r="AA7" s="1" t="s">
-        <v>17</v>
-      </c>
       <c r="AB7" s="1">
         <v>0</v>
       </c>
       <c r="AC7" s="1">
-        <v>423</v>
+        <v>24</v>
       </c>
       <c r="AD7" s="1" t="s">
         <v>123</v>
@@ -1697,16 +1697,16 @@
         <v>123</v>
       </c>
       <c r="AJ7" s="1" t="s">
-        <v>122</v>
+        <v>44</v>
       </c>
       <c r="AK7" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AL7" s="1">
         <v>0</v>
       </c>
       <c r="AM7" s="1">
-        <v>539</v>
+        <v>341</v>
       </c>
       <c r="AN7" s="1" t="s">
         <v>123</v>
@@ -1726,186 +1726,186 @@
     </row>
     <row r="8" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>46</v>
+        <v>100</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C8" s="1">
+        <v>0</v>
+      </c>
+      <c r="D8" s="1">
+        <v>239</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="1">
+        <v>0</v>
+      </c>
+      <c r="I8" s="1">
+        <v>204</v>
+      </c>
+      <c r="J8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K8" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="L8" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="M8" s="1">
+        <v>0</v>
+      </c>
+      <c r="N8" s="1">
+        <v>227</v>
+      </c>
+      <c r="O8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P8" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="Q8" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="R8" s="1">
+        <v>0</v>
+      </c>
+      <c r="S8" s="1">
+        <v>66</v>
+      </c>
+      <c r="T8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U8" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="V8" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="W8" s="1">
+        <v>0</v>
+      </c>
+      <c r="X8" s="1">
+        <v>352</v>
+      </c>
+      <c r="Y8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z8" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="AA8" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="AB8" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC8" s="1">
+        <v>423</v>
+      </c>
+      <c r="AD8" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE8" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="AF8" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>550</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H8" s="1">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1">
-        <v>120</v>
-      </c>
-      <c r="J8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K8" s="1" t="s">
-        <v>102</v>
-      </c>
-      <c r="L8" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="M8" s="1">
-        <v>0</v>
-      </c>
-      <c r="N8" s="1">
-        <v>292</v>
-      </c>
-      <c r="O8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P8" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="Q8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="R8" s="1">
-        <v>0</v>
-      </c>
-      <c r="S8" s="1">
-        <v>446</v>
-      </c>
-      <c r="T8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U8" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="V8" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="W8" s="1">
-        <v>0</v>
-      </c>
-      <c r="X8" s="1">
-        <v>334</v>
-      </c>
-      <c r="Y8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z8" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="AA8" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="AB8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC8" s="1">
-        <v>0</v>
-      </c>
-      <c r="AD8" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE8" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="AF8" s="1" t="s">
-        <v>15</v>
-      </c>
       <c r="AG8" s="1">
         <v>0</v>
       </c>
       <c r="AH8" s="1">
-        <v>348</v>
+        <v>451</v>
       </c>
       <c r="AI8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ8" s="1" t="s">
-        <v>63</v>
+        <v>116</v>
       </c>
       <c r="AK8" s="1" t="s">
-        <v>24</v>
+        <v>13</v>
       </c>
       <c r="AL8" s="1">
         <v>0</v>
       </c>
       <c r="AM8" s="1">
-        <v>253</v>
+        <v>510</v>
       </c>
       <c r="AN8" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO8" s="1" t="s">
-        <v>35</v>
+        <v>99</v>
       </c>
       <c r="AP8" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="AQ8" s="1">
         <v>0</v>
       </c>
       <c r="AR8" s="1">
-        <v>452</v>
+        <v>335</v>
       </c>
     </row>
     <row r="9" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>100</v>
+        <v>74</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>24</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1">
         <v>0</v>
       </c>
       <c r="D9" s="1">
-        <v>237</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>14</v>
+        <v>66</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>15</v>
+        <v>40</v>
       </c>
       <c r="H9" s="1">
         <v>0</v>
       </c>
       <c r="I9" s="1">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="J9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>38</v>
+        <v>16</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="M9" s="1">
         <v>0</v>
       </c>
       <c r="N9" s="1">
-        <v>382</v>
+        <v>392</v>
       </c>
       <c r="O9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P9" s="1" t="s">
-        <v>18</v>
+        <v>77</v>
       </c>
       <c r="Q9" s="1" t="s">
         <v>15</v>
@@ -1914,13 +1914,13 @@
         <v>0</v>
       </c>
       <c r="S9" s="1">
-        <v>177</v>
+        <v>245</v>
       </c>
       <c r="T9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U9" s="1" t="s">
-        <v>95</v>
+        <v>19</v>
       </c>
       <c r="V9" s="1" t="s">
         <v>15</v>
@@ -1929,162 +1929,162 @@
         <v>0</v>
       </c>
       <c r="X9" s="1">
-        <v>297</v>
+        <v>334</v>
       </c>
       <c r="Y9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z9" s="1" t="s">
-        <v>61</v>
+        <v>79</v>
       </c>
       <c r="AA9" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
       <c r="AB9" s="1">
         <v>0</v>
       </c>
       <c r="AC9" s="1">
-        <v>209</v>
+        <v>170</v>
       </c>
       <c r="AD9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE9" s="1" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="AF9" s="1" t="s">
-        <v>34</v>
+        <v>21</v>
       </c>
       <c r="AG9" s="1">
         <v>0</v>
       </c>
       <c r="AH9" s="1">
-        <v>451</v>
+        <v>127</v>
       </c>
       <c r="AI9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ9" s="1" t="s">
-        <v>81</v>
+        <v>107</v>
       </c>
       <c r="AK9" s="1" t="s">
-        <v>54</v>
+        <v>40</v>
       </c>
       <c r="AL9" s="1">
         <v>0</v>
       </c>
       <c r="AM9" s="1">
-        <v>166</v>
+        <v>530</v>
       </c>
       <c r="AN9" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO9" s="1" t="s">
-        <v>73</v>
+        <v>120</v>
       </c>
       <c r="AP9" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="AQ9" s="1">
         <v>0</v>
       </c>
       <c r="AR9" s="1">
-        <v>358</v>
+        <v>432</v>
       </c>
     </row>
     <row r="10" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>119</v>
+        <v>65</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>13</v>
+        <v>29</v>
       </c>
       <c r="C10" s="1">
         <v>0</v>
       </c>
       <c r="D10" s="1">
-        <v>497</v>
+        <v>388</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>37</v>
+        <v>110</v>
       </c>
       <c r="G10" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="H10" s="1">
+        <v>0</v>
+      </c>
+      <c r="I10" s="1">
+        <v>498</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="L10" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M10" s="1">
+        <v>0</v>
+      </c>
+      <c r="N10" s="1">
+        <v>376</v>
+      </c>
+      <c r="O10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P10" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="Q10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="R10" s="1">
+        <v>0</v>
+      </c>
+      <c r="S10" s="1">
+        <v>177</v>
+      </c>
+      <c r="T10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U10" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="V10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>204</v>
-      </c>
-      <c r="J10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="K10" s="1" t="s">
-        <v>67</v>
-      </c>
-      <c r="L10" s="1" t="s">
+      <c r="W10" s="1">
+        <v>0</v>
+      </c>
+      <c r="X10" s="1">
+        <v>455</v>
+      </c>
+      <c r="Y10" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z10" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="AA10" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="M10" s="1">
-        <v>0</v>
-      </c>
-      <c r="N10" s="1">
-        <v>227</v>
-      </c>
-      <c r="O10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="Q10" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="R10" s="1">
-        <v>0</v>
-      </c>
-      <c r="S10" s="1">
-        <v>187</v>
-      </c>
-      <c r="T10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U10" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="V10" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="W10" s="1">
-        <v>0</v>
-      </c>
-      <c r="X10" s="1">
-        <v>352</v>
-      </c>
-      <c r="Y10" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z10" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="AA10" s="1" t="s">
-        <v>24</v>
-      </c>
       <c r="AB10" s="1">
         <v>0</v>
       </c>
       <c r="AC10" s="1">
-        <v>24</v>
+        <v>288</v>
       </c>
       <c r="AD10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE10" s="1" t="s">
-        <v>88</v>
+        <v>32</v>
       </c>
       <c r="AF10" s="1" t="s">
         <v>15</v>
@@ -2093,28 +2093,28 @@
         <v>0</v>
       </c>
       <c r="AH10" s="1">
-        <v>267</v>
+        <v>241</v>
       </c>
       <c r="AI10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ10" s="1" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="AK10" s="1" t="s">
-        <v>24</v>
+        <v>34</v>
       </c>
       <c r="AL10" s="1">
         <v>0</v>
       </c>
       <c r="AM10" s="1">
-        <v>307</v>
+        <v>469</v>
       </c>
       <c r="AN10" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO10" s="1" t="s">
-        <v>99</v>
+        <v>82</v>
       </c>
       <c r="AP10" s="1" t="s">
         <v>23</v>
@@ -2123,27 +2123,27 @@
         <v>0</v>
       </c>
       <c r="AR10" s="1">
-        <v>335</v>
+        <v>515</v>
       </c>
     </row>
     <row r="11" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="C11" s="1">
         <v>0</v>
       </c>
       <c r="D11" s="1">
-        <v>388</v>
+        <v>550</v>
       </c>
       <c r="E11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>92</v>
+        <v>121</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>40</v>
@@ -2152,22 +2152,22 @@
         <v>0</v>
       </c>
       <c r="I11" s="1">
-        <v>446</v>
+        <v>515</v>
       </c>
       <c r="J11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="M11" s="1">
         <v>0</v>
       </c>
       <c r="N11" s="1">
-        <v>392</v>
+        <v>517</v>
       </c>
       <c r="O11" s="1" t="s">
         <v>123</v>
@@ -2188,37 +2188,37 @@
         <v>123</v>
       </c>
       <c r="U11" s="1" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="V11" s="1" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="W11" s="1">
         <v>0</v>
       </c>
       <c r="X11" s="1">
-        <v>205</v>
+        <v>286</v>
       </c>
       <c r="Y11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z11" s="1" t="s">
-        <v>31</v>
+        <v>61</v>
       </c>
       <c r="AA11" s="1" t="s">
-        <v>21</v>
+        <v>34</v>
       </c>
       <c r="AB11" s="1">
         <v>0</v>
       </c>
       <c r="AC11" s="1">
-        <v>432</v>
+        <v>209</v>
       </c>
       <c r="AD11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE11" s="1" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="AF11" s="1" t="s">
         <v>15</v>
@@ -2227,28 +2227,28 @@
         <v>0</v>
       </c>
       <c r="AH11" s="1">
-        <v>241</v>
+        <v>348</v>
       </c>
       <c r="AI11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ11" s="1" t="s">
-        <v>53</v>
+        <v>122</v>
       </c>
       <c r="AK11" s="1" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="AL11" s="1">
         <v>0</v>
       </c>
       <c r="AM11" s="1">
-        <v>123</v>
+        <v>539</v>
       </c>
       <c r="AN11" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO11" s="1" t="s">
-        <v>55</v>
+        <v>64</v>
       </c>
       <c r="AP11" s="1" t="s">
         <v>54</v>
@@ -2257,42 +2257,42 @@
         <v>0</v>
       </c>
       <c r="AR11" s="1">
-        <v>323</v>
+        <v>268</v>
       </c>
     </row>
     <row r="12" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>56</v>
+        <v>109</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C12" s="1">
         <v>0</v>
       </c>
       <c r="D12" s="1">
-        <v>258</v>
+        <v>73</v>
       </c>
       <c r="E12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>121</v>
+        <v>26</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>40</v>
+        <v>23</v>
       </c>
       <c r="H12" s="1">
         <v>0</v>
       </c>
       <c r="I12" s="1">
-        <v>515</v>
+        <v>287</v>
       </c>
       <c r="J12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>58</v>
+        <v>93</v>
       </c>
       <c r="L12" s="1" t="s">
         <v>54</v>
@@ -2301,43 +2301,43 @@
         <v>0</v>
       </c>
       <c r="N12" s="1">
-        <v>376</v>
+        <v>313</v>
       </c>
       <c r="O12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="P12" s="1" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="Q12" s="1" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="R12" s="1">
         <v>0</v>
       </c>
       <c r="S12" s="1">
-        <v>245</v>
+        <v>137</v>
       </c>
       <c r="T12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="U12" s="1" t="s">
-        <v>86</v>
+        <v>30</v>
       </c>
       <c r="V12" s="1" t="s">
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="W12" s="1">
         <v>0</v>
       </c>
       <c r="X12" s="1">
-        <v>286</v>
+        <v>171</v>
       </c>
       <c r="Y12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="Z12" s="1" t="s">
-        <v>87</v>
+        <v>31</v>
       </c>
       <c r="AA12" s="1" t="s">
         <v>21</v>
@@ -2346,66 +2346,66 @@
         <v>0</v>
       </c>
       <c r="AC12" s="1">
-        <v>288</v>
+        <v>432</v>
       </c>
       <c r="AD12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AE12" s="1" t="s">
-        <v>115</v>
+        <v>88</v>
       </c>
       <c r="AF12" s="1" t="s">
-        <v>24</v>
+        <v>15</v>
       </c>
       <c r="AG12" s="1">
         <v>0</v>
       </c>
       <c r="AH12" s="1">
-        <v>346</v>
+        <v>267</v>
       </c>
       <c r="AI12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AJ12" s="1" t="s">
-        <v>116</v>
+        <v>53</v>
       </c>
       <c r="AK12" s="1" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="AL12" s="1">
         <v>0</v>
       </c>
       <c r="AM12" s="1">
-        <v>494</v>
+        <v>123</v>
       </c>
       <c r="AN12" s="1" t="s">
         <v>123</v>
       </c>
       <c r="AO12" s="1" t="s">
-        <v>108</v>
+        <v>55</v>
       </c>
       <c r="AP12" s="1" t="s">
-        <v>13</v>
+        <v>54</v>
       </c>
       <c r="AQ12" s="1">
         <v>0</v>
       </c>
       <c r="AR12" s="1">
-        <v>426</v>
+        <v>323</v>
       </c>
     </row>
     <row r="13" spans="1:44" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C13" s="1">
         <v>0</v>
       </c>
       <c r="D13" s="1">
-        <v>16</v>
+        <v>258</v>
       </c>
       <c r="E13" s="1" t="s">
         <v>123</v>
@@ -2426,106 +2426,106 @@
         <v>123</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>27</v>
+        <v>102</v>
       </c>
       <c r="L13" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1">
+        <v>292</v>
+      </c>
+      <c r="O13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="P13" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="Q13" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="R13" s="1">
+        <v>0</v>
+      </c>
+      <c r="S13" s="1">
+        <v>379</v>
+      </c>
+      <c r="T13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="U13" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="V13" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="W13" s="1">
+        <v>0</v>
+      </c>
+      <c r="X13" s="1">
+        <v>297</v>
+      </c>
+      <c r="Y13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="Z13" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="AA13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="M13" s="1">
-        <v>0</v>
-      </c>
-      <c r="N13" s="1">
-        <v>517</v>
-      </c>
-      <c r="O13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="P13" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="Q13" s="1" t="s">
+      <c r="AB13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AC13" s="1">
+        <v>109</v>
+      </c>
+      <c r="AD13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AE13" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="AF13" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="R13" s="1">
-        <v>0</v>
-      </c>
-      <c r="S13" s="1">
-        <v>380</v>
-      </c>
-      <c r="T13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="U13" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="V13" s="1" t="s">
+      <c r="AG13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AH13" s="1">
+        <v>189</v>
+      </c>
+      <c r="AI13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AJ13" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="AK13" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="W13" s="1">
-        <v>0</v>
-      </c>
-      <c r="X13" s="1">
-        <v>430</v>
-      </c>
-      <c r="Y13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="Z13" s="1" t="s">
-        <v>114</v>
-      </c>
-      <c r="AA13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="AB13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AC13" s="1">
-        <v>297</v>
-      </c>
-      <c r="AD13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AE13" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="AF13" s="1" t="s">
+      <c r="AL13" s="1">
+        <v>0</v>
+      </c>
+      <c r="AM13" s="1">
+        <v>401</v>
+      </c>
+      <c r="AN13" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="AO13" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AP13" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="AG13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AH13" s="1">
-        <v>127</v>
-      </c>
-      <c r="AI13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AJ13" s="1" t="s">
-        <v>107</v>
-      </c>
-      <c r="AK13" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="AL13" s="1">
-        <v>0</v>
-      </c>
-      <c r="AM13" s="1">
-        <v>530</v>
-      </c>
-      <c r="AN13" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="AO13" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="AP13" s="1" t="s">
-        <v>23</v>
-      </c>
       <c r="AQ13" s="1">
         <v>0</v>
       </c>
       <c r="AR13" s="1">
-        <v>515</v>
+        <v>452</v>
       </c>
     </row>
     <row r="14" spans="1:44" x14ac:dyDescent="0.3">
@@ -2650,16 +2650,16 @@
         <v>123</v>
       </c>
       <c r="AO14" s="1" t="s">
-        <v>64</v>
+        <v>73</v>
       </c>
       <c r="AP14" s="1" t="s">
-        <v>54</v>
+        <v>23</v>
       </c>
       <c r="AQ14" s="1">
         <v>0</v>
       </c>
       <c r="AR14" s="1">
-        <v>268</v>
+        <v>358</v>
       </c>
     </row>
     <row r="15" spans="1:44" x14ac:dyDescent="0.3">
@@ -2673,7 +2673,7 @@
         <v>0</v>
       </c>
       <c r="D15" s="1">
-        <v>1991</v>
+        <v>2076</v>
       </c>
       <c r="E15" s="1" t="s">
         <v>123</v>
@@ -2703,7 +2703,7 @@
         <v>0</v>
       </c>
       <c r="N15" s="1">
-        <v>3304</v>
+        <v>3387</v>
       </c>
       <c r="O15" s="1" t="s">
         <v>123</v>
@@ -2733,7 +2733,7 @@
         <v>0</v>
       </c>
       <c r="X15" s="1">
-        <v>2727</v>
+        <v>2747</v>
       </c>
       <c r="Y15" s="1" t="s">
         <v>123</v>
@@ -2748,7 +2748,7 @@
         <v>0</v>
       </c>
       <c r="AC15" s="1">
-        <v>2603</v>
+        <v>2727</v>
       </c>
       <c r="AD15" s="1" t="s">
         <v>123</v>
@@ -2763,7 +2763,7 @@
         <v>0</v>
       </c>
       <c r="AH15" s="1">
-        <v>3235</v>
+        <v>3249</v>
       </c>
       <c r="AI15" s="1" t="s">
         <v>123</v>
@@ -2778,7 +2778,7 @@
         <v>0</v>
       </c>
       <c r="AM15" s="1">
-        <v>3379</v>
+        <v>3432</v>
       </c>
       <c r="AN15" s="1" t="s">
         <v>123</v>
@@ -2793,7 +2793,7 @@
         <v>0</v>
       </c>
       <c r="AR15" s="1">
-        <v>3710</v>
+        <v>4060</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 33
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>293</v>
+        <v>302</v>
       </c>
     </row>
     <row r="5">
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>270</v>
+        <v>356</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>392</v>
+        <v>611</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1527,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="S9">
-        <v>245</v>
+        <v>247</v>
       </c>
       <c r="T9" t="str">
         <v/>
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="Y9" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>177</v>
+        <v>243</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>241</v>
+        <v>305</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>348</v>
+        <v>421</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>137</v>
+        <v>194</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>171</v>
+        <v>219</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -1974,7 +1974,7 @@
         <v>0</v>
       </c>
       <c r="AH12">
-        <v>267</v>
+        <v>282</v>
       </c>
       <c r="AI12" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <v>3613</v>
+        <v>3918</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2331,7 +2331,7 @@
         <v>0</v>
       </c>
       <c r="S15">
-        <v>2481</v>
+        <v>2606</v>
       </c>
       <c r="T15" t="str">
         <v/>
@@ -2346,7 +2346,7 @@
         <v>0</v>
       </c>
       <c r="X15">
-        <v>2855</v>
+        <v>2898</v>
       </c>
       <c r="Y15" t="str">
         <v/>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
       <c r="AH15">
-        <v>3467</v>
+        <v>3619</v>
       </c>
       <c r="AI15" t="str">
         <v/>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="AR15">
-        <v>4078</v>
+        <v>4075</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 34
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>180</v>
+        <v>250</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -991,7 +991,7 @@
         <v>0</v>
       </c>
       <c r="S5">
-        <v>160</v>
+        <v>184</v>
       </c>
       <c r="T5" t="str">
         <v/>
@@ -1170,7 +1170,7 @@
         <v>0</v>
       </c>
       <c r="AH6">
-        <v>0</v>
+        <v>32</v>
       </c>
       <c r="AI6" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>380</v>
+        <v>460</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>553</v>
+        <v>567</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>369</v>
+        <v>424</v>
       </c>
     </row>
     <row r="8">
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>323</v>
+        <v>368</v>
       </c>
     </row>
     <row r="9">
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>530</v>
+        <v>548</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>498</v>
+        <v>546</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>515</v>
+        <v>674</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>517</v>
+        <v>568</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>539</v>
+        <v>595</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>287</v>
+        <v>487</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>379</v>
+        <v>399</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -2093,7 +2093,7 @@
         <v>0</v>
       </c>
       <c r="AC13">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="AD13" t="str">
         <v/>
@@ -2272,7 +2272,7 @@
         <v>0</v>
       </c>
       <c r="AR14">
-        <v>358</v>
+        <v>410</v>
       </c>
     </row>
     <row r="15">
@@ -2301,7 +2301,7 @@
         <v>0</v>
       </c>
       <c r="I15">
-        <v>2560</v>
+        <v>2967</v>
       </c>
       <c r="J15" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v>0</v>
       </c>
       <c r="N15">
-        <v>3918</v>
+        <v>3969</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2331,7 +2331,7 @@
         <v>0</v>
       </c>
       <c r="S15">
-        <v>2606</v>
+        <v>2800</v>
       </c>
       <c r="T15" t="str">
         <v/>
@@ -2361,7 +2361,7 @@
         <v>0</v>
       </c>
       <c r="AC15">
-        <v>2781</v>
+        <v>2785</v>
       </c>
       <c r="AD15" t="str">
         <v/>
@@ -2376,7 +2376,7 @@
         <v>0</v>
       </c>
       <c r="AH15">
-        <v>3619</v>
+        <v>3665</v>
       </c>
       <c r="AI15" t="str">
         <v/>
@@ -2391,7 +2391,7 @@
         <v>0</v>
       </c>
       <c r="AM15">
-        <v>3552</v>
+        <v>3626</v>
       </c>
       <c r="AN15" t="str">
         <v/>
@@ -2406,7 +2406,7 @@
         <v>0</v>
       </c>
       <c r="AR15">
-        <v>4075</v>
+        <v>4227</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 37
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>302</v>
+        <v>350</v>
       </c>
     </row>
     <row r="5">
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>356</v>
+        <v>404</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>460</v>
+        <v>466</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>567</v>
+        <v>703</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>368</v>
+        <v>373</v>
       </c>
     </row>
     <row r="8">
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>611</v>
+        <v>644</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>568</v>
+        <v>655</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>595</v>
+        <v>668</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>487</v>
+        <v>654</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>194</v>
+        <v>208</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>219</v>
+        <v>353</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v/>
       </c>
       <c r="N15">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2614,7 +2614,7 @@
         <v/>
       </c>
       <c r="X17">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="Y17" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -4669,7 +4669,7 @@
         <v/>
       </c>
       <c r="AM32">
-        <v>0</v>
+        <v>40</v>
       </c>
       <c r="AN32" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>410</v>
+        <v>478</v>
       </c>
     </row>
     <row r="39">
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>2610</v>
+        <v>2807</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4187</v>
+        <v>4393</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2466</v>
+        <v>2486</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3003</v>
+        <v>3139</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>3591</v>
+        <v>3781</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>3852</v>
+        <v>3965</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>4816</v>
+        <v>4937</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 38
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="AM6">
-        <v>194</v>
+        <v>210</v>
       </c>
       <c r="AN6" t="str">
         <v/>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>430</v>
+        <v>504</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1393,7 +1393,7 @@
         <v>0</v>
       </c>
       <c r="S8">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="T8" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>448</v>
+        <v>489</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>388</v>
+        <v>498</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>378</v>
+        <v>455</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>286</v>
+        <v>483</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>341</v>
+        <v>429</v>
       </c>
     </row>
     <row r="12">
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>418</v>
+        <v>432</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>167</v>
+        <v>184</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>258</v>
+        <v>342</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>286</v>
+        <v>302</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="N13">
-        <v>294</v>
+        <v>342</v>
       </c>
       <c r="O13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>401</v>
+        <v>418</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>0</v>
+        <v>54</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>0</v>
+        <v>28</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>2350</v>
+        <v>2557</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>2807</v>
+        <v>2851</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4393</v>
+        <v>4532</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2486</v>
+        <v>2496</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3139</v>
+        <v>3451</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>2723</v>
+        <v>2777</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>3965</v>
+        <v>4015</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>4937</v>
+        <v>5025</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 39
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="X3">
-        <v>221</v>
+        <v>235</v>
       </c>
       <c r="Y3" t="str">
         <v/>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>380</v>
+        <v>393</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="AM3">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="AN3" t="str">
         <v/>
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>250</v>
+        <v>432</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>424</v>
+        <v>482</v>
       </c>
     </row>
     <row r="7">
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>383</v>
+        <v>387</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>246</v>
+        <v>281</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>730</v>
+        <v>735</v>
       </c>
     </row>
     <row r="9">
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>548</v>
+        <v>552</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>546</v>
+        <v>694</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>674</v>
+        <v>721</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>399</v>
+        <v>403</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>0</v>
+        <v>96</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="AC23">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="AD23" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>0</v>
+        <v>8</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>0</v>
+        <v>102</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -5011,7 +5011,7 @@
         <v/>
       </c>
       <c r="S35">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>2557</v>
+        <v>2790</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>2851</v>
+        <v>3046</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2496</v>
+        <v>2687</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3451</v>
+        <v>3465</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>2777</v>
+        <v>2800</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4015</v>
+        <v>4022</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5025</v>
+        <v>5088</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 40
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>587</v>
+        <v>619</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>366</v>
+        <v>406</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>515</v>
+        <v>527</v>
       </c>
       <c r="O7" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>212</v>
+        <v>328</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AH8">
-        <v>713</v>
+        <v>765</v>
       </c>
       <c r="AI8" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>135</v>
+        <v>269</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>552</v>
+        <v>623</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>302</v>
+        <v>316</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>539</v>
+        <v>642</v>
       </c>
       <c r="AN10" t="str">
         <v/>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>791</v>
+        <v>892</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>274</v>
+        <v>345</v>
       </c>
       <c r="AD11" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>585</v>
+        <v>641</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>626</v>
+        <v>729</v>
       </c>
     </row>
     <row r="13">
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>0</v>
+        <v>72</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -5115,7 +5115,7 @@
         <v/>
       </c>
       <c r="I36">
-        <v>16</v>
+        <v>60</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>2790</v>
+        <v>2891</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3084</v>
+        <v>3244</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4532</v>
+        <v>4544</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2687</v>
+        <v>2791</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3465</v>
+        <v>3536</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>2800</v>
+        <v>2981</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>3781</v>
+        <v>3967</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4022</v>
+        <v>4125</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5088</v>
+        <v>5191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 41
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>708</v>
+        <v>718</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>70</v>
+        <v>84</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>380</v>
+        <v>544</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>0</v>
+        <v>110</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>832</v>
+        <v>933</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>689</v>
+        <v>842</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>632</v>
+        <v>697</v>
       </c>
       <c r="AN8" t="str">
         <v/>
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>341</v>
+        <v>450</v>
       </c>
       <c r="Y9" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>243</v>
+        <v>253</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>305</v>
+        <v>326</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>421</v>
+        <v>438</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>297</v>
+        <v>536</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="AH18">
-        <v>0</v>
+        <v>76</v>
       </c>
       <c r="AI18" t="str">
         <v/>
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>0</v>
+        <v>38</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -3701,7 +3701,7 @@
         <v/>
       </c>
       <c r="AC25">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="AD25" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>86</v>
+        <v>134</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>48</v>
+        <v>84</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>2891</v>
+        <v>3025</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4544</v>
+        <v>4745</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2791</v>
+        <v>2839</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3536</v>
+        <v>3884</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>2981</v>
+        <v>3159</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>3967</v>
+        <v>4081</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4125</v>
+        <v>4226</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5191</v>
+        <v>5292</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 42
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>432</v>
+        <v>450</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>482</v>
+        <v>494</v>
       </c>
     </row>
     <row r="7">
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>466</v>
+        <v>603</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>703</v>
+        <v>755</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>373</v>
+        <v>395</v>
       </c>
     </row>
     <row r="8">
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>552</v>
+        <v>589</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>694</v>
+        <v>853</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>721</v>
+        <v>799</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>655</v>
+        <v>750</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>668</v>
+        <v>771</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>654</v>
+        <v>684</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>403</v>
+        <v>422</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>96</v>
+        <v>188</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>8</v>
+        <v>131</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>102</v>
+        <v>142</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>54</v>
+        <v>182</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>478</v>
+        <v>536</v>
       </c>
     </row>
     <row r="39">
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3025</v>
+        <v>3157</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3244</v>
+        <v>3511</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4745</v>
+        <v>4840</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>2839</v>
+        <v>3013</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>3159</v>
+        <v>3282</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>4081</v>
+        <v>4261</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4226</v>
+        <v>4366</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5292</v>
+        <v>5384</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 43
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>619</v>
+        <v>701</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="X3">
-        <v>235</v>
+        <v>275</v>
       </c>
       <c r="Y3" t="str">
         <v/>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>393</v>
+        <v>437</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="AM3">
-        <v>347</v>
+        <v>357</v>
       </c>
       <c r="AN3" t="str">
         <v/>
@@ -1036,7 +1036,7 @@
         <v>0</v>
       </c>
       <c r="AH5">
-        <v>502</v>
+        <v>504</v>
       </c>
       <c r="AI5" t="str">
         <v/>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>527</v>
+        <v>605</v>
       </c>
       <c r="O7" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>387</v>
+        <v>441</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AH8">
-        <v>765</v>
+        <v>814</v>
       </c>
       <c r="AI8" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>735</v>
+        <v>886</v>
       </c>
     </row>
     <row r="9">
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>642</v>
+        <v>658</v>
       </c>
       <c r="AN10" t="str">
         <v/>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>892</v>
+        <v>904</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>345</v>
+        <v>519</v>
       </c>
       <c r="AD11" t="str">
         <v/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="AC23">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="AD23" t="str">
         <v/>
@@ -4296,7 +4296,7 @@
         <v/>
       </c>
       <c r="D30">
-        <v>0</v>
+        <v>122</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -5011,7 +5011,7 @@
         <v/>
       </c>
       <c r="S35">
-        <v>5</v>
+        <v>78</v>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -5115,7 +5115,7 @@
         <v/>
       </c>
       <c r="I36">
-        <v>60</v>
+        <v>72</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3157</v>
+        <v>3291</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3511</v>
+        <v>3523</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4840</v>
+        <v>4918</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3013</v>
+        <v>3168</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3884</v>
+        <v>3924</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>3282</v>
+        <v>3504</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>4261</v>
+        <v>4312</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4366</v>
+        <v>4446</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5384</v>
+        <v>5535</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 44
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>350</v>
+        <v>354</v>
       </c>
     </row>
     <row r="5">
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>404</v>
+        <v>490</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>644</v>
+        <v>667</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="Y9" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>253</v>
+        <v>309</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>326</v>
+        <v>375</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>438</v>
+        <v>447</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>208</v>
+        <v>228</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>353</v>
+        <v>474</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>536</v>
+        <v>623</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v/>
       </c>
       <c r="N15">
-        <v>38</v>
+        <v>100</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="AH18">
-        <v>76</v>
+        <v>134</v>
       </c>
       <c r="AI18" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>30</v>
+        <v>166</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>38</v>
+        <v>145</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3291</v>
+        <v>3296</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3523</v>
+        <v>3659</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>4918</v>
+        <v>5089</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3168</v>
+        <v>3351</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>3924</v>
+        <v>4162</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>4312</v>
+        <v>4428</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5535</v>
+        <v>5539</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 4
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>718</v>
+        <v>798</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>84</v>
+        <v>144</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>544</v>
+        <v>679</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>933</v>
+        <v>976</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>842</v>
+        <v>875</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>504</v>
+        <v>602</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>498</v>
+        <v>563</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>483</v>
+        <v>531</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>342</v>
+        <v>466</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>302</v>
+        <v>391</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>418</v>
+        <v>529</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>54</v>
+        <v>138</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>134</v>
+        <v>158</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>84</v>
+        <v>138</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3296</v>
+        <v>3637</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3659</v>
+        <v>3748</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5089</v>
+        <v>5146</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4162</v>
+        <v>4308</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>3504</v>
+        <v>3723</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4446</v>
+        <v>4611</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5539</v>
+        <v>5582</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 46
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>406</v>
+        <v>495</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>603</v>
+        <v>653</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>755</v>
+        <v>869</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>395</v>
+        <v>483</v>
       </c>
     </row>
     <row r="8">
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>328</v>
+        <v>332</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>269</v>
+        <v>381</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>623</v>
+        <v>629</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>316</v>
+        <v>406</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>750</v>
+        <v>828</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>771</v>
+        <v>792</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>684</v>
+        <v>781</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>641</v>
+        <v>682</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>729</v>
+        <v>756</v>
       </c>
     </row>
     <row r="13">
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>72</v>
+        <v>90</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -2406,7 +2406,7 @@
         <v/>
       </c>
       <c r="AR15">
-        <v>0</v>
+        <v>36</v>
       </c>
     </row>
     <row r="16">
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>182</v>
+        <v>363</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>536</v>
+        <v>626</v>
       </c>
     </row>
     <row r="39">
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3748</v>
+        <v>3849</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5146</v>
+        <v>5224</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3351</v>
+        <v>3419</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4308</v>
+        <v>4314</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>3723</v>
+        <v>3943</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>4428</v>
+        <v>4835</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4611</v>
+        <v>4632</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5582</v>
+        <v>5823</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 47
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -902,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>281</v>
+        <v>455</v>
       </c>
       <c r="AI4" t="str">
         <v/>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>115</v>
+        <v>163</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>489</v>
+        <v>537</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>455</v>
+        <v>512</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>309</v>
+        <v>323</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>375</v>
+        <v>407</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="AR10">
-        <v>268</v>
+        <v>272</v>
       </c>
     </row>
     <row r="11">
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>447</v>
+        <v>460</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>429</v>
+        <v>460</v>
       </c>
     </row>
     <row r="12">
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>432</v>
+        <v>524</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>184</v>
+        <v>327</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>623</v>
+        <v>818</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="AH18">
-        <v>134</v>
+        <v>172</v>
       </c>
       <c r="AI18" t="str">
         <v/>
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>145</v>
+        <v>206</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>28</v>
+        <v>46</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3637</v>
+        <v>3685</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3849</v>
+        <v>3867</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5224</v>
+        <v>5373</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3419</v>
+        <v>3494</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4314</v>
+        <v>4557</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>4835</v>
+        <v>5092</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4632</v>
+        <v>4775</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5823</v>
+        <v>5858</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 48
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -738,7 +738,7 @@
         <v>0</v>
       </c>
       <c r="X3">
-        <v>275</v>
+        <v>281</v>
       </c>
       <c r="Y3" t="str">
         <v/>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>437</v>
+        <v>499</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>364</v>
+        <v>424</v>
       </c>
       <c r="AI3" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="AM3">
-        <v>357</v>
+        <v>371</v>
       </c>
       <c r="AN3" t="str">
         <v/>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>490</v>
+        <v>568</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>441</v>
+        <v>505</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>886</v>
+        <v>920</v>
       </c>
     </row>
     <row r="9">
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>667</v>
+        <v>838</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>228</v>
+        <v>240</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>474</v>
+        <v>498</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v/>
       </c>
       <c r="N15">
-        <v>100</v>
+        <v>136</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>166</v>
+        <v>178</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="AC23">
-        <v>6</v>
+        <v>90</v>
       </c>
       <c r="AD23" t="str">
         <v/>
@@ -4296,7 +4296,7 @@
         <v/>
       </c>
       <c r="D30">
-        <v>122</v>
+        <v>163</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -4669,7 +4669,7 @@
         <v/>
       </c>
       <c r="AM32">
-        <v>40</v>
+        <v>118</v>
       </c>
       <c r="AN32" t="str">
         <v/>
@@ -5011,7 +5011,7 @@
         <v/>
       </c>
       <c r="S35">
-        <v>78</v>
+        <v>105</v>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3685</v>
+        <v>3726</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3867</v>
+        <v>3879</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5373</v>
+        <v>5658</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3494</v>
+        <v>3533</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4557</v>
+        <v>4587</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>3943</v>
+        <v>4089</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5092</v>
+        <v>5152</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4775</v>
+        <v>4931</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5858</v>
+        <v>5892</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 49
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>798</v>
+        <v>911</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>144</v>
+        <v>244</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>679</v>
+        <v>763</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>495</v>
+        <v>539</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>976</v>
+        <v>1067</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>875</v>
+        <v>996</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>332</v>
+        <v>378</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>272</v>
+        <v>284</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>697</v>
+        <v>814</v>
       </c>
       <c r="AN8" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>381</v>
+        <v>449</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>629</v>
+        <v>634</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>406</v>
+        <v>453</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>682</v>
+        <v>703</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>756</v>
+        <v>763</v>
       </c>
     </row>
     <row r="13">
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>90</v>
+        <v>299</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -3701,7 +3701,7 @@
         <v/>
       </c>
       <c r="AC25">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="AD25" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>158</v>
+        <v>222</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>138</v>
+        <v>186</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3726</v>
+        <v>3939</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3879</v>
+        <v>3925</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5658</v>
+        <v>5855</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3533</v>
+        <v>3742</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4587</v>
+        <v>4592</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4089</v>
+        <v>4293</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5152</v>
+        <v>5220</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>4931</v>
+        <v>5096</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5892</v>
+        <v>5990</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 50
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>450</v>
+        <v>496</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="AM6">
-        <v>210</v>
+        <v>224</v>
       </c>
       <c r="AN6" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>494</v>
+        <v>620</v>
       </c>
     </row>
     <row r="7">
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>537</v>
+        <v>597</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>589</v>
+        <v>726</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>853</v>
+        <v>873</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>512</v>
+        <v>525</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>799</v>
+        <v>801</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>460</v>
+        <v>544</v>
       </c>
     </row>
     <row r="12">
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>524</v>
+        <v>753</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>327</v>
+        <v>399</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>422</v>
+        <v>512</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>188</v>
+        <v>250</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>131</v>
+        <v>184</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -3775,7 +3775,7 @@
         <v/>
       </c>
       <c r="I26">
-        <v>38</v>
+        <v>76</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>46</v>
+        <v>188</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>142</v>
+        <v>148</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>3939</v>
+        <v>4007</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>3925</v>
+        <v>4127</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>5855</v>
+        <v>6097</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3742</v>
+        <v>3878</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4592</v>
+        <v>4652</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4293</v>
+        <v>4346</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5096</v>
+        <v>5319</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>5990</v>
+        <v>6200</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 51
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>499</v>
+        <v>505</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>424</v>
+        <v>447</v>
       </c>
       <c r="AI3" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="AM3">
-        <v>371</v>
+        <v>381</v>
       </c>
       <c r="AN3" t="str">
         <v/>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>602</v>
+        <v>680</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>505</v>
+        <v>574</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>920</v>
+        <v>967</v>
       </c>
     </row>
     <row r="9">
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>563</v>
+        <v>658</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>531</v>
+        <v>535</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>466</v>
+        <v>494</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>391</v>
+        <v>426</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>529</v>
+        <v>551</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -3165,7 +3165,7 @@
         <v/>
       </c>
       <c r="AC21">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="AD21" t="str">
         <v/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="AC23">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="AD23" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>138</v>
+        <v>231</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -4296,7 +4296,7 @@
         <v/>
       </c>
       <c r="D30">
-        <v>163</v>
+        <v>269</v>
       </c>
       <c r="E30" t="str">
         <v/>
@@ -5011,7 +5011,7 @@
         <v/>
       </c>
       <c r="S35">
-        <v>105</v>
+        <v>119</v>
       </c>
       <c r="T35" t="str">
         <v/>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>25</v>
+        <v>37</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4007</v>
+        <v>4248</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4127</v>
+        <v>4162</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3878</v>
+        <v>3892</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4652</v>
+        <v>4734</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4346</v>
+        <v>4456</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5220</v>
+        <v>5243</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5319</v>
+        <v>5420</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>6200</v>
+        <v>6247</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 52
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>701</v>
+        <v>759</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -1095,7 +1095,7 @@
         <v>0</v>
       </c>
       <c r="I6">
-        <v>179</v>
+        <v>193</v>
       </c>
       <c r="J6" t="str">
         <v/>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>605</v>
+        <v>719</v>
       </c>
       <c r="O7" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>653</v>
+        <v>845</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>869</v>
+        <v>949</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>483</v>
+        <v>586</v>
       </c>
     </row>
     <row r="8">
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AH8">
-        <v>814</v>
+        <v>837</v>
       </c>
       <c r="AI8" t="str">
         <v/>
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>658</v>
+        <v>673</v>
       </c>
       <c r="AN10" t="str">
         <v/>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>904</v>
+        <v>986</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>828</v>
+        <v>865</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>792</v>
+        <v>962</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>781</v>
+        <v>888</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>363</v>
+        <v>508</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>626</v>
+        <v>670</v>
       </c>
     </row>
     <row r="39">
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4248</v>
+        <v>4330</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4162</v>
+        <v>4283</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6097</v>
+        <v>6248</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>3892</v>
+        <v>4142</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5243</v>
+        <v>5491</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5420</v>
+        <v>5605</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>6247</v>
+        <v>6394</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 54
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>496</v>
+        <v>554</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -902,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>455</v>
+        <v>509</v>
       </c>
       <c r="AI4" t="str">
         <v/>
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>354</v>
+        <v>385</v>
       </c>
     </row>
     <row r="5">
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>163</v>
+        <v>191</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>568</v>
+        <v>626</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="AM6">
-        <v>224</v>
+        <v>314</v>
       </c>
       <c r="AN6" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>620</v>
+        <v>757</v>
       </c>
     </row>
     <row r="7">
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>597</v>
+        <v>611</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>838</v>
+        <v>919</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>726</v>
+        <v>758</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>873</v>
+        <v>1060</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>525</v>
+        <v>535</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>323</v>
+        <v>353</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>407</v>
+        <v>409</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1736,7 +1736,7 @@
         <v>0</v>
       </c>
       <c r="AR10">
-        <v>272</v>
+        <v>326</v>
       </c>
     </row>
     <row r="11">
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>801</v>
+        <v>811</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>460</v>
+        <v>583</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>544</v>
+        <v>571</v>
       </c>
     </row>
     <row r="12">
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>753</v>
+        <v>773</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>240</v>
+        <v>274</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>498</v>
+        <v>574</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>399</v>
+        <v>404</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>512</v>
+        <v>514</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>818</v>
+        <v>852</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2316,7 +2316,7 @@
         <v/>
       </c>
       <c r="N15">
-        <v>136</v>
+        <v>268</v>
       </c>
       <c r="O15" t="str">
         <v/>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="AH18">
-        <v>172</v>
+        <v>212</v>
       </c>
       <c r="AI18" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>178</v>
+        <v>267</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>206</v>
+        <v>303</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>250</v>
+        <v>276</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>184</v>
+        <v>234</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -3775,7 +3775,7 @@
         <v/>
       </c>
       <c r="I26">
-        <v>76</v>
+        <v>131</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>188</v>
+        <v>212</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -4669,7 +4669,7 @@
         <v/>
       </c>
       <c r="AM32">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="AN32" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4330</v>
+        <v>4388</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4283</v>
+        <v>4648</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6248</v>
+        <v>6549</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4142</v>
+        <v>4363</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4734</v>
+        <v>4858</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4456</v>
+        <v>4506</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5491</v>
+        <v>5710</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5605</v>
+        <v>5738</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>6394</v>
+        <v>6643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 55
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>505</v>
+        <v>523</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>447</v>
+        <v>461</v>
       </c>
       <c r="AI3" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>539</v>
+        <v>637</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>574</v>
+        <v>700</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>281</v>
+        <v>394</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>378</v>
+        <v>390</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>967</v>
+        <v>988</v>
       </c>
     </row>
     <row r="9">
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>449</v>
+        <v>484</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>634</v>
+        <v>750</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>453</v>
+        <v>477</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>703</v>
+        <v>816</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>763</v>
+        <v>805</v>
       </c>
     </row>
     <row r="13">
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>299</v>
+        <v>381</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -3165,7 +3165,7 @@
         <v/>
       </c>
       <c r="AC21">
-        <v>4</v>
+        <v>54</v>
       </c>
       <c r="AD21" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4388</v>
+        <v>4501</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4648</v>
+        <v>4660</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6549</v>
+        <v>6551</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4363</v>
+        <v>4445</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4858</v>
+        <v>4974</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4506</v>
+        <v>4809</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5710</v>
+        <v>5759</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5738</v>
+        <v>5864</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>6643</v>
+        <v>6706</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 56
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>911</v>
+        <v>952</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>244</v>
+        <v>345</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>763</v>
+        <v>765</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>1067</v>
+        <v>1083</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>996</v>
+        <v>1036</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>845</v>
+        <v>885</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>949</v>
+        <v>1089</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>586</v>
+        <v>694</v>
       </c>
     </row>
     <row r="8">
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>814</v>
+        <v>838</v>
       </c>
       <c r="AN8" t="str">
         <v/>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
       <c r="AR9">
-        <v>515</v>
+        <v>601</v>
       </c>
     </row>
     <row r="10">
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>865</v>
+        <v>924</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>962</v>
+        <v>983</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>888</v>
+        <v>995</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>222</v>
+        <v>230</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>186</v>
+        <v>264</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>508</v>
+        <v>657</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>670</v>
+        <v>758</v>
       </c>
     </row>
     <row r="39">
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4501</v>
+        <v>4643</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4660</v>
+        <v>4767</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6551</v>
+        <v>6658</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4445</v>
+        <v>4485</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4809</v>
+        <v>4811</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>5759</v>
+        <v>6048</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5864</v>
+        <v>5987</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>6706</v>
+        <v>7004</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 57
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>554</v>
+        <v>612</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>757</v>
+        <v>771</v>
       </c>
     </row>
     <row r="7">
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>680</v>
+        <v>732</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>758</v>
+        <v>779</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>658</v>
+        <v>716</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>1060</v>
+        <v>1117</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>811</v>
+        <v>1004</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>535</v>
+        <v>620</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>426</v>
+        <v>485</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>514</v>
+        <v>520</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>551</v>
+        <v>684</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>276</v>
+        <v>358</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3775,7 +3775,7 @@
         <v/>
       </c>
       <c r="I26">
-        <v>131</v>
+        <v>185</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>231</v>
+        <v>365</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4643</v>
+        <v>4787</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>4767</v>
+        <v>5130</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4485</v>
+        <v>4549</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>4974</v>
+        <v>5111</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4811</v>
+        <v>4945</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>5987</v>
+        <v>6141</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>7004</v>
+        <v>7018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 58
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -902,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>509</v>
+        <v>552</v>
       </c>
       <c r="AI4" t="str">
         <v/>
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>191</v>
+        <v>268</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>637</v>
+        <v>671</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>390</v>
+        <v>448</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>286</v>
+        <v>292</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -1527,7 +1527,7 @@
         <v>0</v>
       </c>
       <c r="S9">
-        <v>247</v>
+        <v>279</v>
       </c>
       <c r="T9" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>353</v>
+        <v>375</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>750</v>
+        <v>800</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>477</v>
+        <v>515</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>583</v>
+        <v>742</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>816</v>
+        <v>828</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>805</v>
+        <v>928</v>
       </c>
     </row>
     <row r="13">
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>852</v>
+        <v>956</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>381</v>
+        <v>418</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -2406,7 +2406,7 @@
         <v/>
       </c>
       <c r="AR15">
-        <v>36</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16">
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>303</v>
+        <v>322</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4787</v>
+        <v>4864</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>5130</v>
+        <v>5188</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6658</v>
+        <v>6664</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4549</v>
+        <v>4659</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>5111</v>
+        <v>5265</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>4945</v>
+        <v>5029</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>6048</v>
+        <v>6250</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>7018</v>
+        <v>7197</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 64
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>952</v>
+        <v>1090</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>759</v>
+        <v>968</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>523</v>
+        <v>539</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>461</v>
+        <v>567</v>
       </c>
       <c r="AI3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>345</v>
+        <v>481</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>612</v>
+        <v>674</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>765</v>
+        <v>779</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>385</v>
+        <v>511</v>
       </c>
     </row>
     <row r="5">
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>626</v>
+        <v>698</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>671</v>
+        <v>711</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>1083</v>
+        <v>1135</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>1036</v>
+        <v>1133</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="X6">
-        <v>138</v>
+        <v>167</v>
       </c>
       <c r="Y6" t="str">
         <v/>
@@ -1185,7 +1185,7 @@
         <v>0</v>
       </c>
       <c r="AM6">
-        <v>314</v>
+        <v>332</v>
       </c>
       <c r="AN6" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>771</v>
+        <v>777</v>
       </c>
     </row>
     <row r="7">
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>885</v>
+        <v>899</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>732</v>
+        <v>820</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>1089</v>
+        <v>1111</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>700</v>
+        <v>804</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>694</v>
+        <v>698</v>
       </c>
     </row>
     <row r="8">
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>394</v>
+        <v>421</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>448</v>
+        <v>484</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>292</v>
+        <v>410</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>611</v>
+        <v>659</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AH8">
-        <v>837</v>
+        <v>990</v>
       </c>
       <c r="AI8" t="str">
         <v/>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>838</v>
+        <v>861</v>
       </c>
       <c r="AN8" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>988</v>
+        <v>1080</v>
       </c>
     </row>
     <row r="9">
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>919</v>
+        <v>1036</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>484</v>
+        <v>551</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>716</v>
+        <v>866</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>1117</v>
+        <v>1201</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1646,7 +1646,7 @@
         <v>0</v>
       </c>
       <c r="N10">
-        <v>535</v>
+        <v>547</v>
       </c>
       <c r="O10" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>800</v>
+        <v>810</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>673</v>
+        <v>814</v>
       </c>
       <c r="AN10" t="str">
         <v/>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>986</v>
+        <v>1291</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>1004</v>
+        <v>1128</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>924</v>
+        <v>1029</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>620</v>
+        <v>624</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>519</v>
+        <v>632</v>
       </c>
       <c r="AD11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>983</v>
+        <v>1152</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>571</v>
+        <v>650</v>
       </c>
     </row>
     <row r="12">
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>995</v>
+        <v>1108</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1914,7 +1914,7 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>773</v>
+        <v>1163</v>
       </c>
       <c r="O12" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>274</v>
+        <v>411</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>574</v>
+        <v>616</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>828</v>
+        <v>841</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>404</v>
+        <v>520</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>928</v>
+        <v>934</v>
       </c>
     </row>
     <row r="13">
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>494</v>
+        <v>500</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>485</v>
+        <v>513</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="N13">
-        <v>342</v>
+        <v>354</v>
       </c>
       <c r="O13" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>520</v>
+        <v>592</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>684</v>
+        <v>854</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>418</v>
+        <v>497</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>267</v>
+        <v>315</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -3165,7 +3165,7 @@
         <v/>
       </c>
       <c r="AC21">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="AD21" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>358</v>
+        <v>459</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>234</v>
+        <v>280</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -3775,7 +3775,7 @@
         <v/>
       </c>
       <c r="I26">
-        <v>185</v>
+        <v>311</v>
       </c>
       <c r="J26" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>365</v>
+        <v>375</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>230</v>
+        <v>300</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>212</v>
+        <v>242</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>152</v>
+        <v>186</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -4669,7 +4669,7 @@
         <v/>
       </c>
       <c r="AM32">
-        <v>124</v>
+        <v>179</v>
       </c>
       <c r="AN32" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>264</v>
+        <v>368</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>657</v>
+        <v>671</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>758</v>
+        <v>810</v>
       </c>
     </row>
     <row r="39">
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>4864</v>
+        <v>5761</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>5188</v>
+        <v>5777</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>6664</v>
+        <v>7657</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>4659</v>
+        <v>5232</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>5265</v>
+        <v>5486</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>5029</v>
+        <v>5283</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>6250</v>
+        <v>6612</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>6141</v>
+        <v>7041</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>7197</v>
+        <v>7614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
updated after match 73
</commit_message>
<xml_diff>
--- a/public/data.xlsx
+++ b/public/data.xlsx
@@ -678,7 +678,7 @@
         <v>0</v>
       </c>
       <c r="D3">
-        <v>1090</v>
+        <v>1330</v>
       </c>
       <c r="E3" t="str">
         <v/>
@@ -723,7 +723,7 @@
         <v>0</v>
       </c>
       <c r="S3">
-        <v>968</v>
+        <v>1187</v>
       </c>
       <c r="T3" t="str">
         <v/>
@@ -753,7 +753,7 @@
         <v>0</v>
       </c>
       <c r="AC3">
-        <v>539</v>
+        <v>551</v>
       </c>
       <c r="AD3" t="str">
         <v/>
@@ -768,7 +768,7 @@
         <v>0</v>
       </c>
       <c r="AH3">
-        <v>567</v>
+        <v>699</v>
       </c>
       <c r="AI3" t="str">
         <v/>
@@ -783,7 +783,7 @@
         <v>0</v>
       </c>
       <c r="AM3">
-        <v>381</v>
+        <v>503</v>
       </c>
       <c r="AN3" t="str">
         <v/>
@@ -812,7 +812,7 @@
         <v>0</v>
       </c>
       <c r="D4">
-        <v>481</v>
+        <v>496</v>
       </c>
       <c r="E4" t="str">
         <v/>
@@ -857,7 +857,7 @@
         <v>0</v>
       </c>
       <c r="S4">
-        <v>674</v>
+        <v>766</v>
       </c>
       <c r="T4" t="str">
         <v/>
@@ -887,7 +887,7 @@
         <v>0</v>
       </c>
       <c r="AC4">
-        <v>779</v>
+        <v>906</v>
       </c>
       <c r="AD4" t="str">
         <v/>
@@ -902,7 +902,7 @@
         <v>0</v>
       </c>
       <c r="AH4">
-        <v>552</v>
+        <v>585</v>
       </c>
       <c r="AI4" t="str">
         <v/>
@@ -932,7 +932,7 @@
         <v>0</v>
       </c>
       <c r="AR4">
-        <v>511</v>
+        <v>624</v>
       </c>
     </row>
     <row r="5">
@@ -946,7 +946,7 @@
         <v>0</v>
       </c>
       <c r="D5">
-        <v>268</v>
+        <v>421</v>
       </c>
       <c r="E5" t="str">
         <v/>
@@ -976,7 +976,7 @@
         <v>0</v>
       </c>
       <c r="N5">
-        <v>698</v>
+        <v>705</v>
       </c>
       <c r="O5" t="str">
         <v/>
@@ -1021,7 +1021,7 @@
         <v>0</v>
       </c>
       <c r="AC5">
-        <v>711</v>
+        <v>719</v>
       </c>
       <c r="AD5" t="str">
         <v/>
@@ -1066,7 +1066,7 @@
         <v>0</v>
       </c>
       <c r="AR5">
-        <v>1135</v>
+        <v>1303</v>
       </c>
     </row>
     <row r="6">
@@ -1110,7 +1110,7 @@
         <v>0</v>
       </c>
       <c r="N6">
-        <v>1133</v>
+        <v>1292</v>
       </c>
       <c r="O6" t="str">
         <v/>
@@ -1140,7 +1140,7 @@
         <v>0</v>
       </c>
       <c r="X6">
-        <v>167</v>
+        <v>248</v>
       </c>
       <c r="Y6" t="str">
         <v/>
@@ -1200,7 +1200,7 @@
         <v>0</v>
       </c>
       <c r="AR6">
-        <v>777</v>
+        <v>1063</v>
       </c>
     </row>
     <row r="7">
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="N7">
-        <v>719</v>
+        <v>927</v>
       </c>
       <c r="O7" t="str">
         <v/>
@@ -1259,7 +1259,7 @@
         <v>0</v>
       </c>
       <c r="S7">
-        <v>899</v>
+        <v>1039</v>
       </c>
       <c r="T7" t="str">
         <v/>
@@ -1274,7 +1274,7 @@
         <v>0</v>
       </c>
       <c r="X7">
-        <v>820</v>
+        <v>952</v>
       </c>
       <c r="Y7" t="str">
         <v/>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="AH7">
-        <v>1111</v>
+        <v>1424</v>
       </c>
       <c r="AI7" t="str">
         <v/>
@@ -1319,7 +1319,7 @@
         <v>0</v>
       </c>
       <c r="AM7">
-        <v>804</v>
+        <v>949</v>
       </c>
       <c r="AN7" t="str">
         <v/>
@@ -1334,7 +1334,7 @@
         <v>0</v>
       </c>
       <c r="AR7">
-        <v>698</v>
+        <v>761</v>
       </c>
     </row>
     <row r="8">
@@ -1348,7 +1348,7 @@
         <v>0</v>
       </c>
       <c r="D8">
-        <v>421</v>
+        <v>493</v>
       </c>
       <c r="E8" t="str">
         <v/>
@@ -1363,7 +1363,7 @@
         <v>0</v>
       </c>
       <c r="I8">
-        <v>484</v>
+        <v>566</v>
       </c>
       <c r="J8" t="str">
         <v/>
@@ -1378,7 +1378,7 @@
         <v>0</v>
       </c>
       <c r="N8">
-        <v>410</v>
+        <v>454</v>
       </c>
       <c r="O8" t="str">
         <v/>
@@ -1408,7 +1408,7 @@
         <v>0</v>
       </c>
       <c r="X8">
-        <v>659</v>
+        <v>747</v>
       </c>
       <c r="Y8" t="str">
         <v/>
@@ -1438,7 +1438,7 @@
         <v>0</v>
       </c>
       <c r="AH8">
-        <v>990</v>
+        <v>1419</v>
       </c>
       <c r="AI8" t="str">
         <v/>
@@ -1453,7 +1453,7 @@
         <v>0</v>
       </c>
       <c r="AM8">
-        <v>861</v>
+        <v>1062</v>
       </c>
       <c r="AN8" t="str">
         <v/>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="AR8">
-        <v>1080</v>
+        <v>1204</v>
       </c>
     </row>
     <row r="9">
@@ -1512,7 +1512,7 @@
         <v>0</v>
       </c>
       <c r="N9">
-        <v>1036</v>
+        <v>1038</v>
       </c>
       <c r="O9" t="str">
         <v/>
@@ -1542,7 +1542,7 @@
         <v>0</v>
       </c>
       <c r="X9">
-        <v>480</v>
+        <v>618</v>
       </c>
       <c r="Y9" t="str">
         <v/>
@@ -1572,7 +1572,7 @@
         <v>0</v>
       </c>
       <c r="AH9">
-        <v>551</v>
+        <v>555</v>
       </c>
       <c r="AI9" t="str">
         <v/>
@@ -1587,7 +1587,7 @@
         <v>0</v>
       </c>
       <c r="AM9">
-        <v>779</v>
+        <v>1078</v>
       </c>
       <c r="AN9" t="str">
         <v/>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
       <c r="AR9">
-        <v>601</v>
+        <v>741</v>
       </c>
     </row>
     <row r="10">
@@ -1616,7 +1616,7 @@
         <v>0</v>
       </c>
       <c r="D10">
-        <v>866</v>
+        <v>972</v>
       </c>
       <c r="E10" t="str">
         <v/>
@@ -1631,7 +1631,7 @@
         <v>0</v>
       </c>
       <c r="I10">
-        <v>1201</v>
+        <v>1313</v>
       </c>
       <c r="J10" t="str">
         <v/>
@@ -1661,7 +1661,7 @@
         <v>0</v>
       </c>
       <c r="S10">
-        <v>375</v>
+        <v>443</v>
       </c>
       <c r="T10" t="str">
         <v/>
@@ -1676,7 +1676,7 @@
         <v>0</v>
       </c>
       <c r="X10">
-        <v>810</v>
+        <v>812</v>
       </c>
       <c r="Y10" t="str">
         <v/>
@@ -1691,7 +1691,7 @@
         <v>0</v>
       </c>
       <c r="AC10">
-        <v>515</v>
+        <v>617</v>
       </c>
       <c r="AD10" t="str">
         <v/>
@@ -1706,7 +1706,7 @@
         <v>0</v>
       </c>
       <c r="AH10">
-        <v>409</v>
+        <v>552</v>
       </c>
       <c r="AI10" t="str">
         <v/>
@@ -1721,7 +1721,7 @@
         <v>0</v>
       </c>
       <c r="AM10">
-        <v>814</v>
+        <v>933</v>
       </c>
       <c r="AN10" t="str">
         <v/>
@@ -1750,7 +1750,7 @@
         <v>0</v>
       </c>
       <c r="D11">
-        <v>1291</v>
+        <v>1722</v>
       </c>
       <c r="E11" t="str">
         <v/>
@@ -1765,7 +1765,7 @@
         <v>0</v>
       </c>
       <c r="I11">
-        <v>1128</v>
+        <v>1248</v>
       </c>
       <c r="J11" t="str">
         <v/>
@@ -1780,7 +1780,7 @@
         <v>0</v>
       </c>
       <c r="N11">
-        <v>1029</v>
+        <v>1276</v>
       </c>
       <c r="O11" t="str">
         <v/>
@@ -1810,7 +1810,7 @@
         <v>0</v>
       </c>
       <c r="X11">
-        <v>624</v>
+        <v>660</v>
       </c>
       <c r="Y11" t="str">
         <v/>
@@ -1825,7 +1825,7 @@
         <v>0</v>
       </c>
       <c r="AC11">
-        <v>632</v>
+        <v>751</v>
       </c>
       <c r="AD11" t="str">
         <v/>
@@ -1840,7 +1840,7 @@
         <v>0</v>
       </c>
       <c r="AH11">
-        <v>742</v>
+        <v>791</v>
       </c>
       <c r="AI11" t="str">
         <v/>
@@ -1855,7 +1855,7 @@
         <v>0</v>
       </c>
       <c r="AM11">
-        <v>1152</v>
+        <v>1530</v>
       </c>
       <c r="AN11" t="str">
         <v/>
@@ -1870,7 +1870,7 @@
         <v>0</v>
       </c>
       <c r="AR11">
-        <v>650</v>
+        <v>696</v>
       </c>
     </row>
     <row r="12">
@@ -1899,7 +1899,7 @@
         <v>0</v>
       </c>
       <c r="I12">
-        <v>1108</v>
+        <v>1416</v>
       </c>
       <c r="J12" t="str">
         <v/>
@@ -1929,7 +1929,7 @@
         <v>0</v>
       </c>
       <c r="S12">
-        <v>411</v>
+        <v>421</v>
       </c>
       <c r="T12" t="str">
         <v/>
@@ -1944,7 +1944,7 @@
         <v>0</v>
       </c>
       <c r="X12">
-        <v>616</v>
+        <v>662</v>
       </c>
       <c r="Y12" t="str">
         <v/>
@@ -1959,7 +1959,7 @@
         <v>0</v>
       </c>
       <c r="AC12">
-        <v>841</v>
+        <v>1052</v>
       </c>
       <c r="AD12" t="str">
         <v/>
@@ -1989,7 +1989,7 @@
         <v>0</v>
       </c>
       <c r="AM12">
-        <v>520</v>
+        <v>526</v>
       </c>
       <c r="AN12" t="str">
         <v/>
@@ -2004,7 +2004,7 @@
         <v>0</v>
       </c>
       <c r="AR12">
-        <v>934</v>
+        <v>1081</v>
       </c>
     </row>
     <row r="13">
@@ -2018,7 +2018,7 @@
         <v>0</v>
       </c>
       <c r="D13">
-        <v>500</v>
+        <v>588</v>
       </c>
       <c r="E13" t="str">
         <v/>
@@ -2033,7 +2033,7 @@
         <v>0</v>
       </c>
       <c r="I13">
-        <v>513</v>
+        <v>681</v>
       </c>
       <c r="J13" t="str">
         <v/>
@@ -2048,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="N13">
-        <v>354</v>
+        <v>451</v>
       </c>
       <c r="O13" t="str">
         <v/>
@@ -2063,7 +2063,7 @@
         <v>0</v>
       </c>
       <c r="S13">
-        <v>592</v>
+        <v>637</v>
       </c>
       <c r="T13" t="str">
         <v/>
@@ -2078,7 +2078,7 @@
         <v>0</v>
       </c>
       <c r="X13">
-        <v>956</v>
+        <v>1012</v>
       </c>
       <c r="Y13" t="str">
         <v/>
@@ -2123,7 +2123,7 @@
         <v>0</v>
       </c>
       <c r="AM13">
-        <v>854</v>
+        <v>866</v>
       </c>
       <c r="AN13" t="str">
         <v/>
@@ -2197,7 +2197,7 @@
         <v/>
       </c>
       <c r="S14">
-        <v>497</v>
+        <v>541</v>
       </c>
       <c r="T14" t="str">
         <v/>
@@ -2778,7 +2778,7 @@
         <v/>
       </c>
       <c r="AH18">
-        <v>212</v>
+        <v>312</v>
       </c>
       <c r="AI18" t="str">
         <v/>
@@ -2837,7 +2837,7 @@
         <v/>
       </c>
       <c r="I19">
-        <v>315</v>
+        <v>388</v>
       </c>
       <c r="J19" t="str">
         <v/>
@@ -3001,7 +3001,7 @@
         <v/>
       </c>
       <c r="S20">
-        <v>322</v>
+        <v>354</v>
       </c>
       <c r="T20" t="str">
         <v/>
@@ -3224,7 +3224,7 @@
         <v/>
       </c>
       <c r="D22">
-        <v>459</v>
+        <v>570</v>
       </c>
       <c r="E22" t="str">
         <v/>
@@ -3433,7 +3433,7 @@
         <v/>
       </c>
       <c r="AC23">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="AD23" t="str">
         <v/>
@@ -3567,7 +3567,7 @@
         <v/>
       </c>
       <c r="AC24">
-        <v>280</v>
+        <v>290</v>
       </c>
       <c r="AD24" t="str">
         <v/>
@@ -3969,7 +3969,7 @@
         <v/>
       </c>
       <c r="AC27">
-        <v>375</v>
+        <v>465</v>
       </c>
       <c r="AD27" t="str">
         <v/>
@@ -4058,7 +4058,7 @@
         <v/>
       </c>
       <c r="N28">
-        <v>300</v>
+        <v>444</v>
       </c>
       <c r="O28" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I29">
-        <v>242</v>
+        <v>252</v>
       </c>
       <c r="J29" t="str">
         <v/>
@@ -4430,7 +4430,7 @@
         <v/>
       </c>
       <c r="D31">
-        <v>186</v>
+        <v>228</v>
       </c>
       <c r="E31" t="str">
         <v/>
@@ -4803,7 +4803,7 @@
         <v/>
       </c>
       <c r="AM33">
-        <v>368</v>
+        <v>443</v>
       </c>
       <c r="AN33" t="str">
         <v/>
@@ -4922,7 +4922,7 @@
         <v/>
       </c>
       <c r="AH34">
-        <v>671</v>
+        <v>865</v>
       </c>
       <c r="AI34" t="str">
         <v/>
@@ -5115,7 +5115,7 @@
         <v/>
       </c>
       <c r="I36">
-        <v>72</v>
+        <v>323</v>
       </c>
       <c r="J36" t="str">
         <v/>
@@ -5234,7 +5234,7 @@
         <v/>
       </c>
       <c r="D37">
-        <v>41</v>
+        <v>184</v>
       </c>
       <c r="E37" t="str">
         <v/>
@@ -5488,7 +5488,7 @@
         <v/>
       </c>
       <c r="AR38">
-        <v>810</v>
+        <v>999</v>
       </c>
     </row>
     <row r="39">
@@ -6306,7 +6306,7 @@
         <v>0</v>
       </c>
       <c r="D45">
-        <v>5761</v>
+        <v>7162</v>
       </c>
       <c r="E45" t="str">
         <v/>
@@ -6321,7 +6321,7 @@
         <v>0</v>
       </c>
       <c r="I45">
-        <v>5777</v>
+        <v>6901</v>
       </c>
       <c r="J45" t="str">
         <v/>
@@ -6336,7 +6336,7 @@
         <v>0</v>
       </c>
       <c r="N45">
-        <v>7657</v>
+        <v>8565</v>
       </c>
       <c r="O45" t="str">
         <v/>
@@ -6351,7 +6351,7 @@
         <v>0</v>
       </c>
       <c r="S45">
-        <v>5232</v>
+        <v>5882</v>
       </c>
       <c r="T45" t="str">
         <v/>
@@ -6366,7 +6366,7 @@
         <v>0</v>
       </c>
       <c r="X45">
-        <v>5486</v>
+        <v>6065</v>
       </c>
       <c r="Y45" t="str">
         <v/>
@@ -6381,7 +6381,7 @@
         <v>0</v>
       </c>
       <c r="AC45">
-        <v>5283</v>
+        <v>5976</v>
       </c>
       <c r="AD45" t="str">
         <v/>
@@ -6396,7 +6396,7 @@
         <v>0</v>
       </c>
       <c r="AH45">
-        <v>6612</v>
+        <v>8009</v>
       </c>
       <c r="AI45" t="str">
         <v/>
@@ -6411,7 +6411,7 @@
         <v>0</v>
       </c>
       <c r="AM45">
-        <v>7041</v>
+        <v>8398</v>
       </c>
       <c r="AN45" t="str">
         <v/>
@@ -6560,7 +6560,7 @@
         <v>0</v>
       </c>
       <c r="AR46">
-        <v>7614</v>
+        <v>8890</v>
       </c>
     </row>
   </sheetData>

</xml_diff>